<commit_message>
Complete Phase 1: pagination, file upload, order state machine, inventory alerts
- Add server-side pagination to coupon, wishlist, address, cart, category
  active, and buyer projects endpoints (all now use parsePagination/
  buildPaginatedResponse)
- Add low-stock alerts endpoint (GET /api/products/low-stock) with
  configurable threshold
- Add inventory summary endpoint (GET /api/products/inventory-summary)
  with stock stats and total value
- Update Gantt chart to reflect Phase 1 completion (4/4 items done):
  pagination, file upload middleware, order workflow state machine,
  inventory decrement + alerts
- Overall project completion updated from ~60% to ~68%

https://claude.ai/code/session_01A26UNumk6irmZbm82xEdCk
</commit_message>
<xml_diff>
--- a/MaterialKing_Gantt_Chart.xlsx
+++ b/MaterialKing_Gantt_Chart.xlsx
@@ -53,10 +53,10 @@
       <color rgb="00006100"/>
     </font>
     <font>
-      <color rgb="009C6500"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="009C6500"/>
     </font>
     <font>
       <b val="1"/>
@@ -137,14 +137,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -173,12 +173,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00ED7D31"/>
         <bgColor rgb="00ED7D31"/>
       </patternFill>
@@ -201,6 +195,12 @@
         <bgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -221,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -259,32 +259,31 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -669,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 16 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  6.4 weeks remaining</t>
+          <t>Generated: 21 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  5.7 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1869,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>BACKEND - PENDING (must complete by Apr 30)</t>
+          <t>BACKEND - PHASE 1 COMPLETED (Mar 21)</t>
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
@@ -1888,14 +1887,14 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Product search/filter/sort DONE. Server-side pagination (page/offset/total) MISSING across all endpoints</t>
+          <t>Full pagination across ALL endpoints (products, orders, brands, categories, vendors, zones, buyers, dealers, coupons, wishlist, addresses, cart)</t>
         </is>
       </c>
     </row>
@@ -1910,21 +1909,21 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Status fields exist (pending→confirmed→dispatched→delivered); NO transition validation logic</t>
+          <t>Full state machine: pending→confirmed→processing→shipped→delivered, transition validation, stock restore on cancel</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>Inventory Management (stock decrement)</t>
+          <t>Inventory Management (stock decrement + alerts)</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -1932,14 +1931,14 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>stock_qty field exists; NO auto-decrement on order, NO low-stock alerts</t>
+          <t>Auto-decrement on order, FOR UPDATE locking, restore on cancel, low-stock alerts API, inventory summary endpoint</t>
         </is>
       </c>
     </row>
@@ -1954,43 +1953,31 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>No multer, no S3 config, no upload routes. Images stored as URLs only</t>
+          <t>Multer disk storage, single/multiple upload, file type validation, 10MB limit, /api/upload endpoints</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>Payment Integration (Razorpay)</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>No payment gateway code. Only COD supported</t>
-        </is>
-      </c>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>BACKEND - PENDING (must complete by Apr 30)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Invoice Generation (PDF)</t>
+          <t>Payment Integration (Razorpay)</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -1998,21 +1985,21 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C67" s="9" t="inlineStr">
+      <c r="C67" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>No PDF generation library or templates</t>
+          <t>No payment gateway code. Only COD supported</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Pricing Tiers / Discount Structures</t>
+          <t>Invoice Generation (PDF)</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -2022,19 +2009,19 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
+          <t>No PDF generation library or templates</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking</t>
+          <t>Pricing Tiers / Discount Structures</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -2042,21 +2029,21 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C69" s="8" t="inlineStr">
+      <c r="C69" s="9" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Basic date fields; no tracking numbers or logistics API</t>
+          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>Reporting / Analytics APIs</t>
+          <t>Delivery Tracking</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -2066,73 +2053,73 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>No sales reports, trend analytics, export APIs</t>
+          <t>Basic date fields; no tracking numbers or logistics API</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
+          <t>Reporting / Analytics APIs</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>No sales reports, trend analytics, export APIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
           <t>Notifications (Email/SMS)</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="C71" s="9" t="inlineStr">
+      <c r="C72" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="D72" s="6" t="inlineStr">
         <is>
           <t>No nodemailer/twilio integration</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>FRONTEND - PENDING (must complete by Apr 30)</t>
         </is>
       </c>
-      <c r="B72" s="5" t="n"/>
-      <c r="C72" s="5" t="n"/>
-      <c r="D72" s="5" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Module UI</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>Stock levels, alerts, reorder points dashboard</t>
-        </is>
-      </c>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="5" t="n"/>
+      <c r="D73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>Payment Module UI</t>
+          <t>Inventory Module UI</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -2140,21 +2127,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C74" s="9" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Payment processing screens (Razorpay integration)</t>
+          <t>Stock levels, alerts, reorder points dashboard</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Invoice Module UI</t>
+          <t>Payment Module UI</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
@@ -2162,21 +2149,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C75" s="9" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>View/download invoices as PDF</t>
+          <t>Payment processing screens (Razorpay integration)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking UI</t>
+          <t>Invoice Module UI</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
@@ -2184,21 +2171,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
+      <c r="C76" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Track order delivery status with timeline</t>
+          <t>View/download invoices as PDF</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>Reporting / Dashboard Charts</t>
+          <t>Delivery Tracking UI</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
@@ -2206,21 +2193,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C77" s="9" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Sales summary, top products, dealer analytics with charts</t>
+          <t>Track order delivery status with timeline</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+          <t>Reporting / Dashboard Charts</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -2228,21 +2215,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C78" s="9" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Different dashboards per role</t>
+          <t>Sales summary, top products, dealer analytics with charts</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Products File Upload UI</t>
+          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
@@ -2250,21 +2237,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C79" s="9" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Image upload in product forms (needs Multer backend)</t>
+          <t>Different dashboards per role</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>Responsive Design / Mobile</t>
+          <t>Products File Upload UI</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -2274,47 +2261,70 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Desktop works; mobile nav exists but needs polish</t>
+          <t>Image upload in product forms (needs Multer backend)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
+          <t>Responsive Design / Mobile</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Desktop works; mobile nav exists but needs polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
           <t>Admin Dashboard Charts</t>
         </is>
       </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>Stats cards done; no charts/graphs, no date-range analytics</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="A61:D61"/>
     <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A73:D73"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A66:D66"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2363,7 +2373,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 8 weeks  |  REMAINING: 6.4 weeks  |  Deadline: 30 Apr 2026</t>
+          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 8 weeks  |  REMAINING: 5.7 weeks  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3320,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>PHASE 1 REMAINING (Mar 16-23) ⚡ THIS WEEK</t>
+          <t>PHASE 1 REMAINING (Mar 16-23) ✅ COMPLETED</t>
         </is>
       </c>
       <c r="B23" s="5" t="n"/>
@@ -3335,7 +3345,7 @@
       <c r="U23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Server-side Pagination (all endpoints)</t>
         </is>
@@ -3367,7 +3377,11 @@
       <c r="L24" s="17" t="n"/>
       <c r="M24" s="17" t="n"/>
       <c r="N24" s="17" t="n"/>
-      <c r="O24" s="19" t="n"/>
+      <c r="O24" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P24" s="17" t="n"/>
       <c r="Q24" s="17" t="n"/>
       <c r="R24" s="17" t="n"/>
@@ -3376,7 +3390,7 @@
       <c r="U24" s="17" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>File Upload Middleware (Multer/S3)</t>
         </is>
@@ -3408,7 +3422,11 @@
       <c r="L25" s="17" t="n"/>
       <c r="M25" s="17" t="n"/>
       <c r="N25" s="17" t="n"/>
-      <c r="O25" s="19" t="n"/>
+      <c r="O25" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P25" s="17" t="n"/>
       <c r="Q25" s="17" t="n"/>
       <c r="R25" s="17" t="n"/>
@@ -3417,7 +3435,7 @@
       <c r="U25" s="17" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>Order Workflow State Machine</t>
         </is>
@@ -3449,7 +3467,11 @@
       <c r="L26" s="17" t="n"/>
       <c r="M26" s="17" t="n"/>
       <c r="N26" s="17" t="n"/>
-      <c r="O26" s="19" t="n"/>
+      <c r="O26" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P26" s="17" t="n"/>
       <c r="Q26" s="17" t="n"/>
       <c r="R26" s="17" t="n"/>
@@ -3458,7 +3480,7 @@
       <c r="U26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Inventory Decrement on Order + Alerts</t>
         </is>
@@ -3490,7 +3512,11 @@
       <c r="L27" s="17" t="n"/>
       <c r="M27" s="17" t="n"/>
       <c r="N27" s="17" t="n"/>
-      <c r="O27" s="19" t="n"/>
+      <c r="O27" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P27" s="17" t="n"/>
       <c r="Q27" s="17" t="n"/>
       <c r="R27" s="17" t="n"/>
@@ -3557,12 +3583,12 @@
       <c r="K29" s="17" t="n"/>
       <c r="L29" s="17" t="n"/>
       <c r="M29" s="17" t="n"/>
-      <c r="N29" s="20" t="inlineStr">
+      <c r="N29" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O29" s="20" t="inlineStr">
+      <c r="O29" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3606,7 +3632,7 @@
       <c r="K30" s="17" t="n"/>
       <c r="L30" s="17" t="n"/>
       <c r="M30" s="17" t="n"/>
-      <c r="N30" s="20" t="inlineStr">
+      <c r="N30" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3651,7 +3677,7 @@
       <c r="K31" s="17" t="n"/>
       <c r="L31" s="17" t="n"/>
       <c r="M31" s="17" t="n"/>
-      <c r="N31" s="20" t="inlineStr">
+      <c r="N31" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3696,7 +3722,7 @@
       <c r="K32" s="17" t="n"/>
       <c r="L32" s="17" t="n"/>
       <c r="M32" s="17" t="n"/>
-      <c r="N32" s="20" t="inlineStr">
+      <c r="N32" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3741,12 +3767,12 @@
       <c r="K33" s="17" t="n"/>
       <c r="L33" s="17" t="n"/>
       <c r="M33" s="17" t="n"/>
-      <c r="N33" s="20" t="inlineStr">
+      <c r="N33" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O33" s="20" t="inlineStr">
+      <c r="O33" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3790,12 +3816,12 @@
       <c r="K34" s="17" t="n"/>
       <c r="L34" s="17" t="n"/>
       <c r="M34" s="17" t="n"/>
-      <c r="N34" s="20" t="inlineStr">
+      <c r="N34" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O34" s="20" t="inlineStr">
+      <c r="O34" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3839,12 +3865,12 @@
       <c r="K35" s="17" t="n"/>
       <c r="L35" s="17" t="n"/>
       <c r="M35" s="17" t="n"/>
-      <c r="N35" s="20" t="inlineStr">
+      <c r="N35" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O35" s="20" t="inlineStr">
+      <c r="O35" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3888,12 +3914,12 @@
       <c r="K36" s="17" t="n"/>
       <c r="L36" s="17" t="n"/>
       <c r="M36" s="17" t="n"/>
-      <c r="N36" s="20" t="inlineStr">
+      <c r="N36" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O36" s="20" t="inlineStr">
+      <c r="O36" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3939,7 +3965,7 @@
       <c r="M37" s="17" t="n"/>
       <c r="N37" s="17" t="n"/>
       <c r="O37" s="18" t="n"/>
-      <c r="P37" s="21" t="n"/>
+      <c r="P37" s="20" t="n"/>
       <c r="Q37" s="17" t="n"/>
       <c r="R37" s="17" t="n"/>
       <c r="S37" s="17" t="n"/>
@@ -3980,7 +4006,7 @@
       <c r="M38" s="17" t="n"/>
       <c r="N38" s="17" t="n"/>
       <c r="O38" s="18" t="n"/>
-      <c r="P38" s="21" t="n"/>
+      <c r="P38" s="20" t="n"/>
       <c r="Q38" s="17" t="n"/>
       <c r="R38" s="17" t="n"/>
       <c r="S38" s="17" t="n"/>
@@ -4021,8 +4047,8 @@
       <c r="M39" s="17" t="n"/>
       <c r="N39" s="17" t="n"/>
       <c r="O39" s="18" t="n"/>
-      <c r="P39" s="21" t="n"/>
-      <c r="Q39" s="21" t="n"/>
+      <c r="P39" s="20" t="n"/>
+      <c r="Q39" s="20" t="n"/>
       <c r="R39" s="17" t="n"/>
       <c r="S39" s="17" t="n"/>
       <c r="T39" s="17" t="n"/>
@@ -4063,7 +4089,7 @@
       <c r="N40" s="17" t="n"/>
       <c r="O40" s="18" t="n"/>
       <c r="P40" s="17" t="n"/>
-      <c r="Q40" s="21" t="n"/>
+      <c r="Q40" s="20" t="n"/>
       <c r="R40" s="17" t="n"/>
       <c r="S40" s="17" t="n"/>
       <c r="T40" s="17" t="n"/>
@@ -4132,7 +4158,7 @@
       <c r="O42" s="18" t="n"/>
       <c r="P42" s="17" t="n"/>
       <c r="Q42" s="17" t="n"/>
-      <c r="R42" s="22" t="n"/>
+      <c r="R42" s="21" t="n"/>
       <c r="S42" s="17" t="n"/>
       <c r="T42" s="17" t="n"/>
       <c r="U42" s="17" t="n"/>
@@ -4173,7 +4199,7 @@
       <c r="O43" s="18" t="n"/>
       <c r="P43" s="17" t="n"/>
       <c r="Q43" s="17" t="n"/>
-      <c r="R43" s="22" t="n"/>
+      <c r="R43" s="21" t="n"/>
       <c r="S43" s="17" t="n"/>
       <c r="T43" s="17" t="n"/>
       <c r="U43" s="17" t="n"/>
@@ -4215,7 +4241,7 @@
       <c r="P44" s="17" t="n"/>
       <c r="Q44" s="17" t="n"/>
       <c r="R44" s="17" t="n"/>
-      <c r="S44" s="22" t="n"/>
+      <c r="S44" s="21" t="n"/>
       <c r="T44" s="17" t="n"/>
       <c r="U44" s="17" t="n"/>
     </row>
@@ -4255,8 +4281,8 @@
       <c r="O45" s="18" t="n"/>
       <c r="P45" s="17" t="n"/>
       <c r="Q45" s="17" t="n"/>
-      <c r="R45" s="22" t="n"/>
-      <c r="S45" s="22" t="n"/>
+      <c r="R45" s="21" t="n"/>
+      <c r="S45" s="21" t="n"/>
       <c r="T45" s="17" t="n"/>
       <c r="U45" s="17" t="n"/>
     </row>
@@ -4296,7 +4322,7 @@
       <c r="O46" s="18" t="n"/>
       <c r="P46" s="17" t="n"/>
       <c r="Q46" s="17" t="n"/>
-      <c r="R46" s="22" t="n"/>
+      <c r="R46" s="21" t="n"/>
       <c r="S46" s="17" t="n"/>
       <c r="T46" s="17" t="n"/>
       <c r="U46" s="17" t="n"/>
@@ -4337,8 +4363,8 @@
       <c r="O47" s="18" t="n"/>
       <c r="P47" s="17" t="n"/>
       <c r="Q47" s="17" t="n"/>
-      <c r="R47" s="22" t="n"/>
-      <c r="S47" s="22" t="n"/>
+      <c r="R47" s="21" t="n"/>
+      <c r="S47" s="21" t="n"/>
       <c r="T47" s="17" t="n"/>
       <c r="U47" s="17" t="n"/>
     </row>
@@ -4379,7 +4405,7 @@
       <c r="P48" s="17" t="n"/>
       <c r="Q48" s="17" t="n"/>
       <c r="R48" s="17" t="n"/>
-      <c r="S48" s="22" t="n"/>
+      <c r="S48" s="21" t="n"/>
       <c r="T48" s="17" t="n"/>
       <c r="U48" s="17" t="n"/>
     </row>
@@ -4448,7 +4474,7 @@
       <c r="Q50" s="17" t="n"/>
       <c r="R50" s="17" t="n"/>
       <c r="S50" s="17" t="n"/>
-      <c r="T50" s="23" t="n"/>
+      <c r="T50" s="22" t="n"/>
       <c r="U50" s="17" t="n"/>
     </row>
     <row r="51">
@@ -4489,7 +4515,7 @@
       <c r="Q51" s="17" t="n"/>
       <c r="R51" s="17" t="n"/>
       <c r="S51" s="17" t="n"/>
-      <c r="T51" s="23" t="n"/>
+      <c r="T51" s="22" t="n"/>
       <c r="U51" s="17" t="n"/>
     </row>
     <row r="52">
@@ -4530,7 +4556,7 @@
       <c r="Q52" s="17" t="n"/>
       <c r="R52" s="17" t="n"/>
       <c r="S52" s="17" t="n"/>
-      <c r="T52" s="23" t="n"/>
+      <c r="T52" s="22" t="n"/>
       <c r="U52" s="17" t="n"/>
     </row>
     <row r="53">
@@ -4571,7 +4597,7 @@
       <c r="Q53" s="17" t="n"/>
       <c r="R53" s="17" t="n"/>
       <c r="S53" s="17" t="n"/>
-      <c r="T53" s="23" t="n"/>
+      <c r="T53" s="22" t="n"/>
       <c r="U53" s="17" t="n"/>
     </row>
     <row r="54">
@@ -4613,7 +4639,7 @@
       <c r="R54" s="17" t="n"/>
       <c r="S54" s="17" t="n"/>
       <c r="T54" s="17" t="n"/>
-      <c r="U54" s="23" t="n"/>
+      <c r="U54" s="22" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -4654,91 +4680,91 @@
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="17" t="n"/>
       <c r="T55" s="17" t="n"/>
-      <c r="U55" s="23" t="n"/>
+      <c r="U55" s="22" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="24" t="inlineStr">
-        <is>
-          <t>▲ TODAY (Mar 16, 2026) — 6.4 weeks to deadline</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="n"/>
-      <c r="C56" s="25" t="n"/>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="25" t="n"/>
-      <c r="F56" s="25" t="n"/>
-      <c r="G56" s="25" t="n"/>
-      <c r="H56" s="25" t="n"/>
-      <c r="I56" s="25" t="n"/>
-      <c r="J56" s="25" t="n"/>
-      <c r="K56" s="25" t="n"/>
-      <c r="L56" s="25" t="n"/>
-      <c r="M56" s="25" t="n"/>
-      <c r="N56" s="25" t="n"/>
-      <c r="O56" s="26" t="inlineStr">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>▲ TODAY (Mar 21, 2026) — 5.7 weeks to deadline</t>
+        </is>
+      </c>
+      <c r="B56" s="24" t="n"/>
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="24" t="n"/>
+      <c r="G56" s="24" t="n"/>
+      <c r="H56" s="24" t="n"/>
+      <c r="I56" s="24" t="n"/>
+      <c r="J56" s="24" t="n"/>
+      <c r="K56" s="24" t="n"/>
+      <c r="L56" s="24" t="n"/>
+      <c r="M56" s="24" t="n"/>
+      <c r="N56" s="24" t="n"/>
+      <c r="O56" s="25" t="inlineStr">
         <is>
           <t>▲ NOW</t>
         </is>
       </c>
-      <c r="P56" s="25" t="n"/>
-      <c r="Q56" s="25" t="n"/>
-      <c r="R56" s="25" t="n"/>
-      <c r="S56" s="25" t="n"/>
-      <c r="T56" s="25" t="n"/>
-      <c r="U56" s="25" t="n"/>
+      <c r="P56" s="24" t="n"/>
+      <c r="Q56" s="24" t="n"/>
+      <c r="R56" s="24" t="n"/>
+      <c r="S56" s="24" t="n"/>
+      <c r="T56" s="24" t="n"/>
+      <c r="U56" s="24" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="inlineStr">
+      <c r="A58" s="26" t="inlineStr">
         <is>
           <t>LEGEND:</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="n"/>
-      <c r="B59" s="29" t="inlineStr">
+      <c r="A59" s="27" t="n"/>
+      <c r="B59" s="28" t="inlineStr">
         <is>
           <t>Completed (Jan 22 - Mar 10)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="30" t="n"/>
-      <c r="B60" s="29" t="inlineStr">
-        <is>
-          <t>Phase 1: Foundation (Mar 10-23) — mostly DONE</t>
+      <c r="A60" s="29" t="n"/>
+      <c r="B60" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1: Foundation (Mar 10-23) — COMPLETED</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="31" t="n"/>
-      <c r="B61" s="29" t="inlineStr">
+      <c r="A61" s="30" t="n"/>
+      <c r="B61" s="28" t="inlineStr">
         <is>
           <t>Phase 2: Core CRUD (Mar 24 - Apr 6) — frontend DONE, backend partial</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="32" t="n"/>
-      <c r="B62" s="29" t="inlineStr">
+      <c r="A62" s="31" t="n"/>
+      <c r="B62" s="28" t="inlineStr">
         <is>
           <t>Phase 3: Business Logic &amp; Dashboard (Apr 7-20)</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="33" t="n"/>
-      <c r="B63" s="29" t="inlineStr">
+      <c r="A63" s="32" t="n"/>
+      <c r="B63" s="28" t="inlineStr">
         <is>
           <t>Phase 4: Polish &amp; Launch (Apr 21-30)</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="34" t="n"/>
-      <c r="B64" s="29" t="inlineStr">
-        <is>
-          <t>TODAY marker (Mar 16)</t>
+      <c r="A64" s="33" t="n"/>
+      <c r="B64" s="28" t="inlineStr">
+        <is>
+          <t>TODAY marker (Mar 21)</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4779,7 +4805,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>PROJECT SUMMARY</t>
         </is>
@@ -4788,23 +4814,23 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Start: 22 Jan 2026  |  Today: 16 Mar 2026  |  Deadline: 30 Apr 2026</t>
+          <t>Start: 22 Jan 2026  |  Today: 21 Mar 2026  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr"/>
-      <c r="B4" s="36" t="inlineStr"/>
-      <c r="C4" s="36" t="inlineStr"/>
+      <c r="A4" s="35" t="inlineStr"/>
+      <c r="B4" s="35" t="inlineStr"/>
+      <c r="C4" s="35" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>TIMELINE</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr"/>
-      <c r="C5" s="37" t="inlineStr"/>
+      <c r="B5" s="36" t="inlineStr"/>
+      <c r="C5" s="36" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -4827,7 +4853,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>16 Mar 2026</t>
+          <t>21 Mar 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -4849,7 +4875,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>6.4 weeks remaining</t>
+          <t>5.7 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -4871,22 +4897,22 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr"/>
-      <c r="B10" s="36" t="inlineStr"/>
-      <c r="C10" s="36" t="inlineStr"/>
+      <c r="A10" s="35" t="inlineStr"/>
+      <c r="B10" s="35" t="inlineStr"/>
+      <c r="C10" s="35" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>COMPLETION STATUS</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C11" s="37" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -4912,447 +4938,464 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Backend Features Pending</t>
+          <t>Backend Features Completed (Phase 1)</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>7 features</t>
+          <t>4 features</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Pagination, File Upload, Payments, Invoices, Reporting, Notifications, Pricing Tiers</t>
+          <t>Pagination (all endpoints), File Upload (Multer), Order State Machine, Inventory Decrement + Alerts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Backend Features Partial</t>
+          <t>Backend Features Pending</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>3 features</t>
+          <t>4 features</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Order Workflow (needs transition validation), Inventory (needs decrement), Delivery Tracking</t>
+          <t>Payments (Razorpay), Invoices (PDF), Reporting APIs, Notifications (Email/SMS)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Frontend Completed</t>
+          <t>Backend Features Partial</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>48 items</t>
+          <t>2 features</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>All admin CRUD (9 modules), all storefront pages (11), buyer account (4), foundation (10), UI components (4), nav/footer</t>
+          <t>Pricing Tiers (coupon done, tier logic pending), Delivery Tracking (basic fields, no logistics API)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>Frontend Completed</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>48 items</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>All admin CRUD (9 modules), all storefront pages (11), buyer account (4), foundation (10), UI components (4), nav/footer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>Frontend Pending</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>8 items</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Inventory UI, Payment UI, Invoice UI, Delivery UI, Dashboard Charts, Role-based Dashboards, File Upload UI, Responsive polish</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="36" t="inlineStr"/>
-      <c r="B17" s="36" t="inlineStr"/>
-      <c r="C17" s="36" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr"/>
+      <c r="B18" s="35" t="inlineStr"/>
+      <c r="C18" s="35" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>Overall Completion</t>
         </is>
       </c>
-      <c r="B18" s="38" t="inlineStr">
-        <is>
-          <t>~60%</t>
-        </is>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>Backend CRUD + Frontend CRUD + Storefront all done. Remaining: business logic backends + specialized UIs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="36" t="inlineStr"/>
-      <c r="B19" s="36" t="inlineStr"/>
-      <c r="C19" s="36" t="inlineStr"/>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>~68%</t>
+        </is>
+      </c>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>Backend CRUD + Phase 1 features + Frontend CRUD + Storefront all done. Remaining: business logic backends + specialized UIs.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="37" t="inlineStr">
+      <c r="A20" s="35" t="inlineStr"/>
+      <c r="B20" s="35" t="inlineStr"/>
+      <c r="C20" s="35" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>RISK ASSESSMENT</t>
         </is>
       </c>
-      <c r="B20" s="37" t="inlineStr"/>
-      <c r="C20" s="37" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Schedule Risk</t>
-        </is>
-      </c>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Ahead of schedule on frontend. ~40% work in 6.4 weeks. Manageable with focus.</t>
-        </is>
-      </c>
+      <c r="B21" s="36" t="inlineStr"/>
+      <c r="C21" s="36" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Critical Path</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Payments + Invoices + Inventory</t>
+          <t>Schedule Risk</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>MEDIUM-LOW</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>These depend on each other — must start this week</t>
+          <t>Phase 1 complete. ~32% work in 5.7 weeks. On track with focused sprints.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Parallel Tracks Needed</t>
+          <t>Critical Path</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Payments + Invoices</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Backend features (pagination, upload, payments) + Frontend UIs simultaneously</t>
+          <t>These depend on each other — next priority in Phase 2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>Parallel Tracks Needed</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Backend features (payments, invoices) + Frontend UIs simultaneously</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>Recommended Action</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>FOCUSED SPRINTS</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Tackle P0 items (pagination, upload, state machine, inventory) this week</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="36" t="inlineStr"/>
-      <c r="B25" s="36" t="inlineStr"/>
-      <c r="C25" s="36" t="inlineStr"/>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Start Phase 2: Razorpay + Invoice PDF + Pricing Tiers next week</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="37" t="inlineStr">
+      <c r="A26" s="35" t="inlineStr"/>
+      <c r="B26" s="35" t="inlineStr"/>
+      <c r="C26" s="35" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
         <is>
           <t>PHASE PLAN (REMAINING)</t>
         </is>
       </c>
-      <c r="B26" s="37" t="inlineStr">
+      <c r="B27" s="36" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>Focus</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Phase 1 Remaining</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Mar 16-23 (1 wk)</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Pagination, File Upload, Order State Machine, Inventory Decrement</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Phase 2 Remaining</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Mar 24 - Apr 6 (2 wks)</t>
+          <t>Mar 16-23 (1 wk)</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation, Product file upload UI</t>
+          <t>COMPLETED: Pagination, File Upload, Order State Machine, Inventory Decrement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Phase 3: Business Logic</t>
+          <t>Phase 2 Remaining</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Apr 7-20 (2 wks)</t>
+          <t>Mar 24 - Apr 6 (2 wks)</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Inventory UI, Payment UI, Invoice UI, Dashboard charts, Reporting APIs, Delivery tracking, Notifications</t>
+          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation, Product file upload UI</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t>Phase 3: Business Logic</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Apr 7-20 (2 wks)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Inventory UI, Payment UI, Invoice UI, Dashboard charts, Reporting APIs, Delivery tracking, Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>Phase 4: Polish &amp; Launch</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Apr 21-30 (1.5 wks)</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Role-based dashboards, responsive design, testing, UAT, deployment</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="36" t="inlineStr"/>
-      <c r="B31" s="36" t="inlineStr"/>
-      <c r="C31" s="36" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="37" t="inlineStr">
+      <c r="A32" s="35" t="inlineStr"/>
+      <c r="B32" s="35" t="inlineStr"/>
+      <c r="C32" s="35" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
         <is>
           <t>WHAT WAS DONE AHEAD OF SCHEDULE</t>
         </is>
       </c>
-      <c r="B32" s="37" t="inlineStr"/>
-      <c r="C32" s="37" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>All Admin CRUD UIs (9 modules)</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Phase 2 → Done in Phase 1</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard</t>
-        </is>
-      </c>
+      <c r="B33" s="36" t="inlineStr"/>
+      <c r="C33" s="36" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>All Storefront Pages (11 pages)</t>
+          <t>All Admin CRUD UIs (9 modules)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Phase 2-3 → Done in Phase 1</t>
+          <t>Phase 2 → Done in Phase 1</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Home, Products, Detail, Cart, Checkout, Confirmation, Categories, About, Contact + Header/Footer</t>
+          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Buyer Account (4 pages)</t>
+          <t>All Storefront Pages (11 pages)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Phase 3 → Done in Phase 1</t>
+          <t>Phase 2-3 → Done in Phase 1</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>My Account, My Orders, Addresses, Wishlist</t>
+          <t>Home, Products, Detail, Cart, Checkout, Confirmation, Categories, About, Contact + Header/Footer</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
+          <t>Buyer Account (4 pages)</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Phase 3 → Done in Phase 1</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>My Account, My Orders, Addresses, Wishlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
           <t>Cart + Wishlist + Coupon APIs</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Not in plan → Done</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Server-side cart, wishlist, coupon validation — bonus features</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="36" t="inlineStr"/>
-      <c r="B37" s="36" t="inlineStr"/>
-      <c r="C37" s="36" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" s="37" t="inlineStr">
+      <c r="A38" s="35" t="inlineStr"/>
+      <c r="B38" s="35" t="inlineStr"/>
+      <c r="C38" s="35" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="36" t="inlineStr">
         <is>
           <t>TEAM ALLOCATION (suggested for remaining)</t>
         </is>
       </c>
-      <c r="B38" s="37" t="inlineStr"/>
-      <c r="C38" s="37" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Dev 1 (Frontend Lead)</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>File Upload UI → Role-based Dashboards → Responsive polish</t>
-        </is>
-      </c>
+      <c r="B39" s="36" t="inlineStr"/>
+      <c r="C39" s="36" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Dev 2 (Frontend)</t>
+          <t>Dev 1 (Frontend Lead)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr"/>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Dashboard Charts → Reporting UI → Integration testing</t>
+          <t>File Upload UI → Role-based Dashboards → Responsive polish</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Dev 3 (Backend + Frontend)</t>
+          <t>Dev 2 (Frontend)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr"/>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Pagination → Invoice PDF backend → Reporting APIs</t>
+          <t>Dashboard Charts → Reporting UI → Integration testing</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Dev 4 (Backend Lead)</t>
+          <t>Dev 3 (Backend + Frontend)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr"/>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>File Upload Multer → Inventory decrement → Notifications</t>
+          <t>Pagination → Invoice PDF backend → Reporting APIs</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Dev 5 (Frontend)</t>
+          <t>Dev 4 (Backend Lead)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Inventory UI → Dashboard charts → Responsive design</t>
+          <t>File Upload Multer → Inventory decrement → Notifications</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Dev 6 (Frontend)</t>
+          <t>Dev 5 (Frontend)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr"/>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Payment UI → Invoice UI → Role-based views</t>
+          <t>Inventory UI → Dashboard charts → Responsive design</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Dev 7 (Backend)</t>
+          <t>Dev 6 (Frontend)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr"/>
       <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Payment UI → Invoice UI → Role-based views</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Dev 7 (Backend)</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Order State Machine → Razorpay → Delivery tracking</t>
         </is>

</xml_diff>

<commit_message>
Update Gantt chart: refresh all statuses to Mar 21, 2026
- Phase 1 Remaining: all 4 items marked DONE (pagination, file upload, order state machine, inventory)
- Phase 2: Coupons, Admin Users, and File Upload UI marked DONE
- Backend completed count: 17 → 21 modules
- Frontend completed count: 48 → 54 items
- Overall completion: ~60% → ~70%
- Schedule risk downgraded: MEDIUM → LOW-MEDIUM
- Updated team allocation for remaining work
- Remaining: 4 backend features + 7 frontend UIs + testing/deployment in 5.7 weeks

https://claude.ai/code/session_0147TWQhvrJuRoRZiqK4BvoS
</commit_message>
<xml_diff>
--- a/MaterialKing_Gantt_Chart.xlsx
+++ b/MaterialKing_Gantt_Chart.xlsx
@@ -53,10 +53,10 @@
       <color rgb="00006100"/>
     </font>
     <font>
-      <color rgb="009C6500"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="009C6500"/>
     </font>
     <font>
       <b val="1"/>
@@ -137,14 +137,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -173,12 +173,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00ED7D31"/>
         <bgColor rgb="00ED7D31"/>
       </patternFill>
@@ -201,6 +195,12 @@
         <bgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -221,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -259,32 +259,31 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -669,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 16 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  6.4 weeks remaining</t>
+          <t>Generated: 21 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  5.7 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -698,7 +697,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>BACKEND - COMPLETED (Jan 22 - Mar 10, ~7 weeks)</t>
+          <t>BACKEND - COMPLETED (Jan 22 - Mar 21)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -972,7 +971,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Address API</t>
+          <t>Admin Users API</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -987,14 +986,14 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>CRUD for user addresses with default address support</t>
+          <t>CRUD for admin user management with role assignment</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>DB Schema (15+ tables) + Seed Script</t>
+          <t>Address API</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -1009,14 +1008,14 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Full schema with migration patches</t>
+          <t>CRUD for user addresses with default address support</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Validation &amp; Error Middleware</t>
+          <t>DB Schema (15+ tables) + Seed Script</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1031,51 +1030,63 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Request validation middleware</t>
+          <t>Full schema with migration patches</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>Validation &amp; Error Middleware</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Request validation middleware</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>Role-based Access Control</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Admin, dealer, buyer, vendor roles</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - FOUNDATION (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Vite + React 19 + TypeScript</t>
+          <t>Server-side Pagination (all endpoints)</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1085,19 +1096,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Project scaffolded and running</t>
+          <t>page/offset/total across all list endpoints — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Tailwind CSS Config (custom MK theme)</t>
+          <t>File Upload Middleware (Multer)</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1107,19 +1118,19 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>mk-red, mk-gray palette, Montserrat font</t>
+          <t>Multer middleware for Tech Data Sheet PDF uploads — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>BrowserRouter + Route Definitions</t>
+          <t>Order Workflow State Machine</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1129,19 +1140,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Full route tree: public, admin, account sections</t>
+          <t>Transition validation (pending→confirmed→dispatched→delivered) — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>React Query (QueryClientProvider)</t>
+          <t>Inventory Decrement on Order + Alerts</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1151,36 +1162,24 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Configured with retry:1, staleTime:30s</t>
+          <t>Auto-decrement stock on order, low-stock validation — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Axios API Client + Token Refresh</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Auto-refresh on 401, concurrent request queue</t>
-        </is>
-      </c>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - FOUNDATION (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>AuthContext + useAuth hook</t>
+          <t>Vite + React 19 + TypeScript</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -1195,14 +1194,14 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Login/logout/updateUser/isAdmin, auto-load on mount</t>
+          <t>Project scaffolded and running</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Protected Routes / Route Guards</t>
+          <t>Tailwind CSS Config (custom MK theme)</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -1217,14 +1216,14 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>ProtectedRoute component with loading spinner</t>
+          <t>mk-red, mk-gray palette, Montserrat font</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>API Service Layer (13 modules)</t>
+          <t>BrowserRouter + Route Definitions</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -1239,14 +1238,14 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>product, category, brand, vendor, zone, dealer, buyer, order, auth, cart, coupon, wishlist, address</t>
+          <t>Full route tree: public, admin, account sections</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Login Page</t>
+          <t>React Query (QueryClientProvider)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -1261,14 +1260,14 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Email/password login with validation</t>
+          <t>Configured with retry:1, staleTime:30s</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Register Page</t>
+          <t>Axios API Client + Token Refresh</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1283,24 +1282,36 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>User registration with role selection</t>
+          <t>Auto-refresh on 401, concurrent request queue</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - ADMIN CRUD MODULES (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>AuthContext + useAuth hook</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Login/logout/updateUser/isAdmin, auto-load on mount</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Admin Dashboard</t>
+          <t>Protected Routes / Route Guards</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1315,14 +1326,14 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Stats cards (orders, revenue, products, buyers, dealers) + recent orders table</t>
+          <t>ProtectedRoute component with loading spinner</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Products Module (list + forms)</t>
+          <t>API Service Layer (13 modules)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1337,14 +1348,14 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Full CRUD with 4-tab form (basic, dimensions, attributes, packaging)</t>
+          <t>product, category, brand, vendor, zone, dealer, buyer, order, auth, cart, coupon, wishlist, address, adminUser</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Brands Module (list + forms)</t>
+          <t>Login Page</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1359,14 +1370,14 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>CRUD with DataTable + FormModal</t>
+          <t>Email/password login with validation</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Categories Module (list + forms)</t>
+          <t>Register Page</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1381,36 +1392,24 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>CRUD with parent/child hierarchy</t>
+          <t>User registration with role selection</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Vendors Module (list + forms)</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>CRUD with DataTable + FormModal</t>
-        </is>
-      </c>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - ADMIN CRUD MODULES (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Zones Module (list + forms)</t>
+          <t>Admin Dashboard</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1425,14 +1424,14 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>CRUD with DataTable + FormModal</t>
+          <t>Stats cards (orders, revenue, products, buyers, dealers) + recent orders table</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Buyers Module (list + forms)</t>
+          <t>Products Module (list + forms)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -1447,14 +1446,14 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>CRUD with DataTable + FormModal</t>
+          <t>Full CRUD with 4-tab form (basic, dimensions, attributes, packaging)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Dealers Module (list + forms)</t>
+          <t>Brands Module (list + forms)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -1476,7 +1475,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Orders Module (list + detail)</t>
+          <t>Categories Module (list + forms)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -1491,14 +1490,14 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Admin order management with status updates</t>
+          <t>CRUD with parent/child hierarchy</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Reusable UI Components</t>
+          <t>Vendors Module (list + forms)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -1513,24 +1512,36 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>DataTable, FormField, FormModal, StatusBadge</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - STOREFRONT PAGES (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Zones Module (list + forms)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>CRUD with DataTable + FormModal</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Public Header + Nav with Category Hover Dropdowns</t>
+          <t>Buyers Module (list + forms)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -1545,14 +1556,14 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>7 merged categories, hover subcategory menus, linked to products</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Public Footer</t>
+          <t>Dealers Module (list + forms)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -1567,14 +1578,14 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Footer with links</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Home Page</t>
+          <t>Orders Module (list + detail)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -1589,14 +1600,14 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Hero section + featured products</t>
+          <t>Admin order management with status updates</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Products List Page</t>
+          <t>Coupons Module (list + forms)</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -1611,14 +1622,14 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Filters (category, brand, price range, search, sort)</t>
+          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Product Detail Page</t>
+          <t>Admin Users Module (list + forms)</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -1633,14 +1644,14 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Product info tabs, wishlist, add to cart</t>
+          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Categories Page</t>
+          <t>Reusable UI Components</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -1655,14 +1666,14 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Category grid with subcategory tags</t>
+          <t>DataTable, FormField, FormModal, StatusBadge</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Cart Page</t>
+          <t>Products File Upload UI</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -1677,36 +1688,24 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Cart items, coupon apply, tax/shipping calc</t>
+          <t>Tech Data Sheet PDF upload in product forms — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>Checkout Page</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Address selection, payment method, order placement</t>
-        </is>
-      </c>
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - STOREFRONT PAGES (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Order Confirmation Page</t>
+          <t>Public Header + Nav with Category Hover Dropdowns</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -1721,14 +1720,14 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Post-checkout confirmation (protected)</t>
+          <t>7 merged categories, hover subcategory menus, linked to products</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>About Page</t>
+          <t>Public Footer</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -1743,14 +1742,14 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Static about us page</t>
+          <t>Footer with correct office address</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Contact Page</t>
+          <t>Home Page</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -1765,24 +1764,36 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Contact form</t>
+          <t>Hero section + featured products</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - BUYER ACCOUNT (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Products List Page</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Filters (category, brand, price range, search, sort)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>My Account Page</t>
+          <t>Product Detail Page</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -1797,14 +1808,14 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Profile management</t>
+          <t>Product info tabs, wishlist, add to cart</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>My Orders Page</t>
+          <t>Categories Page</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -1819,14 +1830,14 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Order history with detail view</t>
+          <t>Category grid with subcategory tags</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Addresses Page</t>
+          <t>Cart Page</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -1841,14 +1852,14 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Saved addresses CRUD with default</t>
+          <t>Cart items, coupon apply, tax/shipping calc</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Wishlist Page</t>
+          <t>Checkout Page</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -1863,200 +1874,188 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Wishlist management</t>
+          <t>Address selection, payment method, order placement</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>BACKEND - PENDING (must complete by Apr 30)</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="5" t="n"/>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Order Confirmation Page</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Post-checkout confirmation (protected)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>Search &amp; Filtering + Pagination (server-side)</t>
+          <t>About Page</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Product search/filter/sort DONE. Server-side pagination (page/offset/total) MISSING across all endpoints</t>
+          <t>Static about us page</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>Order Workflow State Machine</t>
+          <t>Contact Page</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Status fields exist (pending→confirmed→dispatched→delivered); NO transition validation logic</t>
+          <t>Contact form with office address</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Management (stock decrement)</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>stock_qty field exists; NO auto-decrement on order, NO low-stock alerts</t>
-        </is>
-      </c>
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - BUYER ACCOUNT (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n"/>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>File Upload Middleware (Multer/S3)</t>
+          <t>My Account Page</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>No multer, no S3 config, no upload routes. Images stored as URLs only</t>
+          <t>Profile management</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Payment Integration (Razorpay)</t>
+          <t>My Orders Page</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>No payment gateway code. Only COD supported</t>
+          <t>Order history with detail view</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Invoice Generation (PDF)</t>
+          <t>Addresses Page</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>No PDF generation library or templates</t>
+          <t>Saved addresses CRUD with default</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Pricing Tiers / Discount Structures</t>
+          <t>Wishlist Page</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
+          <t>Wishlist management</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>Delivery Tracking</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>Basic date fields; no tracking numbers or logistics API</t>
-        </is>
-      </c>
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>BACKEND - PENDING (must complete by Apr 30)</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n"/>
+      <c r="C69" s="5" t="n"/>
+      <c r="D69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>Reporting / Analytics APIs</t>
+          <t>Payment Integration (Razorpay)</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -2064,21 +2063,21 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>No sales reports, trend analytics, export APIs</t>
+          <t>No payment gateway code. Only COD supported</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Notifications (Email/SMS)</t>
+          <t>Invoice Generation (PDF)</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -2086,119 +2085,119 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="C71" s="9" t="inlineStr">
+      <c r="C71" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>No nodemailer/twilio integration</t>
+          <t>No PDF generation library or templates</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - PENDING (must complete by Apr 30)</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="n"/>
-      <c r="C72" s="5" t="n"/>
-      <c r="D72" s="5" t="n"/>
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Pricing Tiers / Discount Structures</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>Inventory Module UI</t>
+          <t>Delivery Tracking</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Stock levels, alerts, reorder points dashboard</t>
+          <t>Basic date fields; no tracking numbers or logistics API</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>Payment Module UI</t>
+          <t>Reporting / Analytics APIs</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Payment processing screens (Razorpay integration)</t>
+          <t>No sales reports, trend analytics, export APIs</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Invoice Module UI</t>
+          <t>Notifications (Email/SMS)</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C75" s="9" t="inlineStr">
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>View/download invoices as PDF</t>
+          <t>No nodemailer/twilio integration</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>Delivery Tracking UI</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Track order delivery status with timeline</t>
-        </is>
-      </c>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - PENDING (must complete by Apr 30)</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="n"/>
+      <c r="C76" s="5" t="n"/>
+      <c r="D76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>Reporting / Dashboard Charts</t>
+          <t>Inventory Module UI</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
@@ -2206,21 +2205,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C77" s="9" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Sales summary, top products, dealer analytics with charts</t>
+          <t>Stock levels, alerts, reorder points dashboard</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+          <t>Payment Module UI</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -2228,21 +2227,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C78" s="9" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Different dashboards per role</t>
+          <t>Payment processing screens (Razorpay integration)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Products File Upload UI</t>
+          <t>Invoice Module UI</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
@@ -2250,21 +2249,21 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C79" s="9" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Image upload in product forms (needs Multer backend)</t>
+          <t>View/download invoices as PDF</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>Responsive Design / Mobile</t>
+          <t>Delivery Tracking UI</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -2274,32 +2273,98 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Desktop works; mobile nav exists but needs polish</t>
+          <t>Track order delivery status with timeline</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
+          <t>Reporting / Dashboard Charts</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Sales summary, top products, dealer analytics with charts</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>Different dashboards per role</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Responsive Design / Mobile</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Desktop works; mobile nav exists but needs polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
           <t>Admin Dashboard Charts</t>
         </is>
       </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D84" s="6" t="inlineStr">
         <is>
           <t>Stats cards done; no charts/graphs, no date-range analytics</t>
         </is>
@@ -2309,13 +2374,13 @@
   <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A64:D64"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A76:D76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2327,7 +2392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U64"/>
+  <dimension ref="A1:U65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2363,7 +2428,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 8 weeks  |  REMAINING: 6.4 weeks  |  Deadline: 30 Apr 2026</t>
+          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 8 weeks  |  REMAINING: 5.7 weeks  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -3308,36 +3373,54 @@
       <c r="U22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 1 REMAINING (Mar 16-23) ⚡ THIS WEEK</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5" t="n"/>
-      <c r="P23" s="5" t="n"/>
-      <c r="Q23" s="5" t="n"/>
-      <c r="R23" s="5" t="n"/>
-      <c r="S23" s="5" t="n"/>
-      <c r="T23" s="5" t="n"/>
-      <c r="U23" s="5" t="n"/>
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Server-side Pagination (all endpoints)</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>46097</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>46103</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="n"/>
+      <c r="I23" s="17" t="n"/>
+      <c r="J23" s="17" t="n"/>
+      <c r="K23" s="17" t="n"/>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="n"/>
+      <c r="N23" s="17" t="n"/>
+      <c r="O23" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P23" s="17" t="n"/>
+      <c r="Q23" s="17" t="n"/>
+      <c r="R23" s="17" t="n"/>
+      <c r="S23" s="17" t="n"/>
+      <c r="T23" s="17" t="n"/>
+      <c r="U23" s="17" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Server-side Pagination (all endpoints)</t>
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>File Upload Middleware (Multer)</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -3347,7 +3430,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 4</t>
         </is>
       </c>
       <c r="D24" s="14" t="n">
@@ -3367,7 +3450,11 @@
       <c r="L24" s="17" t="n"/>
       <c r="M24" s="17" t="n"/>
       <c r="N24" s="17" t="n"/>
-      <c r="O24" s="19" t="n"/>
+      <c r="O24" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P24" s="17" t="n"/>
       <c r="Q24" s="17" t="n"/>
       <c r="R24" s="17" t="n"/>
@@ -3376,9 +3463,9 @@
       <c r="U24" s="17" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>File Upload Middleware (Multer/S3)</t>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Order Workflow State Machine</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -3388,7 +3475,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Dev 4</t>
+          <t>Dev 7</t>
         </is>
       </c>
       <c r="D25" s="14" t="n">
@@ -3408,7 +3495,11 @@
       <c r="L25" s="17" t="n"/>
       <c r="M25" s="17" t="n"/>
       <c r="N25" s="17" t="n"/>
-      <c r="O25" s="19" t="n"/>
+      <c r="O25" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P25" s="17" t="n"/>
       <c r="Q25" s="17" t="n"/>
       <c r="R25" s="17" t="n"/>
@@ -3417,9 +3508,9 @@
       <c r="U25" s="17" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Order Workflow State Machine</t>
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Inventory Decrement on Order + Alerts</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -3429,7 +3520,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Dev 7</t>
+          <t>Dev 4</t>
         </is>
       </c>
       <c r="D26" s="14" t="n">
@@ -3449,7 +3540,11 @@
       <c r="L26" s="17" t="n"/>
       <c r="M26" s="17" t="n"/>
       <c r="N26" s="17" t="n"/>
-      <c r="O26" s="19" t="n"/>
+      <c r="O26" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P26" s="17" t="n"/>
       <c r="Q26" s="17" t="n"/>
       <c r="R26" s="17" t="n"/>
@@ -3458,77 +3553,85 @@
       <c r="U26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Decrement on Order + Alerts</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Dev 4</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>46097</v>
-      </c>
-      <c r="E27" s="14" t="n">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>PHASE 2: CORE MODULES (Mar 24 - Apr 6) — Frontend DONE, Backend in progress</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
+      <c r="L27" s="5" t="n"/>
+      <c r="M27" s="5" t="n"/>
+      <c r="N27" s="5" t="n"/>
+      <c r="O27" s="5" t="n"/>
+      <c r="P27" s="5" t="n"/>
+      <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="5" t="n"/>
+      <c r="S27" s="5" t="n"/>
+      <c r="T27" s="5" t="n"/>
+      <c r="U27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Products Module UI (list + forms + 4 tabs)</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Dev 1</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>46090</v>
+      </c>
+      <c r="E28" s="14" t="n">
         <v>46103</v>
       </c>
-      <c r="F27" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="17" t="n"/>
-      <c r="H27" s="17" t="n"/>
-      <c r="I27" s="17" t="n"/>
-      <c r="J27" s="17" t="n"/>
-      <c r="K27" s="17" t="n"/>
-      <c r="L27" s="17" t="n"/>
-      <c r="M27" s="17" t="n"/>
-      <c r="N27" s="17" t="n"/>
-      <c r="O27" s="19" t="n"/>
-      <c r="P27" s="17" t="n"/>
-      <c r="Q27" s="17" t="n"/>
-      <c r="R27" s="17" t="n"/>
-      <c r="S27" s="17" t="n"/>
-      <c r="T27" s="17" t="n"/>
-      <c r="U27" s="17" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 2: CORE MODULES (Mar 24 - Apr 6)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="5" t="n"/>
-      <c r="P28" s="5" t="n"/>
-      <c r="Q28" s="5" t="n"/>
-      <c r="R28" s="5" t="n"/>
-      <c r="S28" s="5" t="n"/>
-      <c r="T28" s="5" t="n"/>
-      <c r="U28" s="5" t="n"/>
+      <c r="F28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="17" t="n"/>
+      <c r="H28" s="17" t="n"/>
+      <c r="I28" s="17" t="n"/>
+      <c r="J28" s="17" t="n"/>
+      <c r="K28" s="17" t="n"/>
+      <c r="L28" s="17" t="n"/>
+      <c r="M28" s="17" t="n"/>
+      <c r="N28" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O28" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P28" s="17" t="n"/>
+      <c r="Q28" s="17" t="n"/>
+      <c r="R28" s="17" t="n"/>
+      <c r="S28" s="17" t="n"/>
+      <c r="T28" s="17" t="n"/>
+      <c r="U28" s="17" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Products Module UI (list + forms + 4 tabs)</t>
+          <t>Brands + Categories Module UI</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -3538,17 +3641,17 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Dev 1</t>
+          <t>Dev 2</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>46103</v>
+        <v>46096</v>
       </c>
       <c r="F29" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G29" s="17" t="n"/>
       <c r="H29" s="17" t="n"/>
@@ -3557,16 +3660,12 @@
       <c r="K29" s="17" t="n"/>
       <c r="L29" s="17" t="n"/>
       <c r="M29" s="17" t="n"/>
-      <c r="N29" s="20" t="inlineStr">
+      <c r="N29" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O29" s="20" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="O29" s="18" t="n"/>
       <c r="P29" s="17" t="n"/>
       <c r="Q29" s="17" t="n"/>
       <c r="R29" s="17" t="n"/>
@@ -3577,7 +3676,7 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Brands + Categories Module UI</t>
+          <t>Vendors Module UI</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -3587,7 +3686,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Dev 2</t>
+          <t>Dev 5</t>
         </is>
       </c>
       <c r="D30" s="14" t="n">
@@ -3606,7 +3705,7 @@
       <c r="K30" s="17" t="n"/>
       <c r="L30" s="17" t="n"/>
       <c r="M30" s="17" t="n"/>
-      <c r="N30" s="20" t="inlineStr">
+      <c r="N30" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3622,7 +3721,7 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Vendors Module UI</t>
+          <t>Zones Module UI</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -3651,7 +3750,7 @@
       <c r="K31" s="17" t="n"/>
       <c r="L31" s="17" t="n"/>
       <c r="M31" s="17" t="n"/>
-      <c r="N31" s="20" t="inlineStr">
+      <c r="N31" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3667,7 +3766,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Zones Module UI</t>
+          <t>Dealers Module UI</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -3677,17 +3776,17 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Dev 5</t>
+          <t>Dev 6</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>46096</v>
+        <v>46103</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="17" t="n"/>
       <c r="H32" s="17" t="n"/>
@@ -3696,12 +3795,16 @@
       <c r="K32" s="17" t="n"/>
       <c r="L32" s="17" t="n"/>
       <c r="M32" s="17" t="n"/>
-      <c r="N32" s="20" t="inlineStr">
+      <c r="N32" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O32" s="18" t="n"/>
+      <c r="O32" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P32" s="17" t="n"/>
       <c r="Q32" s="17" t="n"/>
       <c r="R32" s="17" t="n"/>
@@ -3712,7 +3815,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Dealers Module UI</t>
+          <t>Buyers Module UI</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -3722,7 +3825,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Dev 6</t>
+          <t>Dev 2</t>
         </is>
       </c>
       <c r="D33" s="14" t="n">
@@ -3741,12 +3844,12 @@
       <c r="K33" s="17" t="n"/>
       <c r="L33" s="17" t="n"/>
       <c r="M33" s="17" t="n"/>
-      <c r="N33" s="20" t="inlineStr">
+      <c r="N33" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O33" s="20" t="inlineStr">
+      <c r="O33" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3761,7 +3864,7 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Buyers Module UI</t>
+          <t>Orders Module UI (admin)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -3771,7 +3874,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Dev 2</t>
+          <t>Dev 1, Dev 2</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
@@ -3790,12 +3893,12 @@
       <c r="K34" s="17" t="n"/>
       <c r="L34" s="17" t="n"/>
       <c r="M34" s="17" t="n"/>
-      <c r="N34" s="20" t="inlineStr">
+      <c r="N34" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O34" s="20" t="inlineStr">
+      <c r="O34" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3810,7 +3913,7 @@
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Orders Module UI (admin)</t>
+          <t>Admin Dashboard (stats + recent orders)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -3820,7 +3923,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Dev 1, Dev 2</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D35" s="14" t="n">
@@ -3839,12 +3942,12 @@
       <c r="K35" s="17" t="n"/>
       <c r="L35" s="17" t="n"/>
       <c r="M35" s="17" t="n"/>
-      <c r="N35" s="20" t="inlineStr">
+      <c r="N35" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O35" s="20" t="inlineStr">
+      <c r="O35" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -3859,7 +3962,7 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Admin Dashboard (stats + recent orders)</t>
+          <t>Coupons Module (both frontends)</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -3869,14 +3972,14 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
-        <v>46090</v>
+        <v>46097</v>
       </c>
       <c r="E36" s="14" t="n">
-        <v>46103</v>
+        <v>46110</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>2</v>
@@ -3888,17 +3991,17 @@
       <c r="K36" s="17" t="n"/>
       <c r="L36" s="17" t="n"/>
       <c r="M36" s="17" t="n"/>
-      <c r="N36" s="20" t="inlineStr">
+      <c r="N36" s="17" t="n"/>
+      <c r="O36" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O36" s="20" t="inlineStr">
+      <c r="P36" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P36" s="17" t="n"/>
       <c r="Q36" s="17" t="n"/>
       <c r="R36" s="17" t="n"/>
       <c r="S36" s="17" t="n"/>
@@ -3906,9 +4009,9 @@
       <c r="U36" s="17" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Products File Upload UI (needs Multer)</t>
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Admin Users Module (both frontends)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -3922,13 +4025,13 @@
         </is>
       </c>
       <c r="D37" s="14" t="n">
-        <v>46104</v>
+        <v>46097</v>
       </c>
       <c r="E37" s="14" t="n">
         <v>46110</v>
       </c>
       <c r="F37" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="17" t="n"/>
       <c r="H37" s="17" t="n"/>
@@ -3938,8 +4041,16 @@
       <c r="L37" s="17" t="n"/>
       <c r="M37" s="17" t="n"/>
       <c r="N37" s="17" t="n"/>
-      <c r="O37" s="18" t="n"/>
-      <c r="P37" s="21" t="n"/>
+      <c r="O37" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P37" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q37" s="17" t="n"/>
       <c r="R37" s="17" t="n"/>
       <c r="S37" s="17" t="n"/>
@@ -3947,26 +4058,26 @@
       <c r="U37" s="17" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Pricing Tiers / Discount Backend</t>
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Products File Upload UI (Tech Data Sheet)</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Dev 4</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D38" s="14" t="n">
-        <v>46104</v>
+        <v>46097</v>
       </c>
       <c r="E38" s="14" t="n">
-        <v>46110</v>
+        <v>46103</v>
       </c>
       <c r="F38" s="15" t="n">
         <v>1</v>
@@ -3979,8 +4090,12 @@
       <c r="L38" s="17" t="n"/>
       <c r="M38" s="17" t="n"/>
       <c r="N38" s="17" t="n"/>
-      <c r="O38" s="18" t="n"/>
-      <c r="P38" s="21" t="n"/>
+      <c r="O38" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P38" s="17" t="n"/>
       <c r="Q38" s="17" t="n"/>
       <c r="R38" s="17" t="n"/>
       <c r="S38" s="17" t="n"/>
@@ -3990,7 +4105,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Payment Integration Backend (Razorpay)</t>
+          <t>Pricing Tiers / Discount Backend</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -4000,17 +4115,17 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Dev 7</t>
+          <t>Dev 4</t>
         </is>
       </c>
       <c r="D39" s="14" t="n">
         <v>46104</v>
       </c>
       <c r="E39" s="14" t="n">
-        <v>46117</v>
+        <v>46110</v>
       </c>
       <c r="F39" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="17" t="n"/>
       <c r="H39" s="17" t="n"/>
@@ -4021,8 +4136,8 @@
       <c r="M39" s="17" t="n"/>
       <c r="N39" s="17" t="n"/>
       <c r="O39" s="18" t="n"/>
-      <c r="P39" s="21" t="n"/>
-      <c r="Q39" s="21" t="n"/>
+      <c r="P39" s="20" t="n"/>
+      <c r="Q39" s="17" t="n"/>
       <c r="R39" s="17" t="n"/>
       <c r="S39" s="17" t="n"/>
       <c r="T39" s="17" t="n"/>
@@ -4031,7 +4146,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Invoice Generation Backend (PDF)</t>
+          <t>Payment Integration Backend (Razorpay)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -4041,17 +4156,17 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 7</t>
         </is>
       </c>
       <c r="D40" s="14" t="n">
-        <v>46111</v>
+        <v>46104</v>
       </c>
       <c r="E40" s="14" t="n">
         <v>46117</v>
       </c>
       <c r="F40" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="17" t="n"/>
       <c r="H40" s="17" t="n"/>
@@ -4062,85 +4177,85 @@
       <c r="M40" s="17" t="n"/>
       <c r="N40" s="17" t="n"/>
       <c r="O40" s="18" t="n"/>
-      <c r="P40" s="17" t="n"/>
-      <c r="Q40" s="21" t="n"/>
+      <c r="P40" s="20" t="n"/>
+      <c r="Q40" s="20" t="n"/>
       <c r="R40" s="17" t="n"/>
       <c r="S40" s="17" t="n"/>
       <c r="T40" s="17" t="n"/>
       <c r="U40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Invoice Generation Backend (PDF)</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="n">
+        <v>46111</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>46117</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="17" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="17" t="n"/>
+      <c r="J41" s="17" t="n"/>
+      <c r="K41" s="17" t="n"/>
+      <c r="L41" s="17" t="n"/>
+      <c r="M41" s="17" t="n"/>
+      <c r="N41" s="17" t="n"/>
+      <c r="O41" s="18" t="n"/>
+      <c r="P41" s="17" t="n"/>
+      <c r="Q41" s="20" t="n"/>
+      <c r="R41" s="17" t="n"/>
+      <c r="S41" s="17" t="n"/>
+      <c r="T41" s="17" t="n"/>
+      <c r="U41" s="17" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>PHASE 3: BUSINESS LOGIC &amp; DASHBOARD (Apr 7 - Apr 20)</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
-      <c r="L41" s="5" t="n"/>
-      <c r="M41" s="5" t="n"/>
-      <c r="N41" s="5" t="n"/>
-      <c r="O41" s="5" t="n"/>
-      <c r="P41" s="5" t="n"/>
-      <c r="Q41" s="5" t="n"/>
-      <c r="R41" s="5" t="n"/>
-      <c r="S41" s="5" t="n"/>
-      <c r="T41" s="5" t="n"/>
-      <c r="U41" s="5" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Module UI (stock levels, alerts)</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Dev 5</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="n">
-        <v>46118</v>
-      </c>
-      <c r="E42" s="14" t="n">
-        <v>46124</v>
-      </c>
-      <c r="F42" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="17" t="n"/>
-      <c r="H42" s="17" t="n"/>
-      <c r="I42" s="17" t="n"/>
-      <c r="J42" s="17" t="n"/>
-      <c r="K42" s="17" t="n"/>
-      <c r="L42" s="17" t="n"/>
-      <c r="M42" s="17" t="n"/>
-      <c r="N42" s="17" t="n"/>
-      <c r="O42" s="18" t="n"/>
-      <c r="P42" s="17" t="n"/>
-      <c r="Q42" s="17" t="n"/>
-      <c r="R42" s="22" t="n"/>
-      <c r="S42" s="17" t="n"/>
-      <c r="T42" s="17" t="n"/>
-      <c r="U42" s="17" t="n"/>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
+      <c r="J42" s="5" t="n"/>
+      <c r="K42" s="5" t="n"/>
+      <c r="L42" s="5" t="n"/>
+      <c r="M42" s="5" t="n"/>
+      <c r="N42" s="5" t="n"/>
+      <c r="O42" s="5" t="n"/>
+      <c r="P42" s="5" t="n"/>
+      <c r="Q42" s="5" t="n"/>
+      <c r="R42" s="5" t="n"/>
+      <c r="S42" s="5" t="n"/>
+      <c r="T42" s="5" t="n"/>
+      <c r="U42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Payment Module UI (Razorpay frontend)</t>
+          <t>Inventory Module UI (stock levels, alerts)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -4150,7 +4265,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Dev 6</t>
+          <t>Dev 5</t>
         </is>
       </c>
       <c r="D43" s="14" t="n">
@@ -4173,7 +4288,7 @@
       <c r="O43" s="18" t="n"/>
       <c r="P43" s="17" t="n"/>
       <c r="Q43" s="17" t="n"/>
-      <c r="R43" s="22" t="n"/>
+      <c r="R43" s="21" t="n"/>
       <c r="S43" s="17" t="n"/>
       <c r="T43" s="17" t="n"/>
       <c r="U43" s="17" t="n"/>
@@ -4181,7 +4296,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Invoice Module UI (view/download PDF)</t>
+          <t>Payment Module UI (Razorpay frontend)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -4195,10 +4310,10 @@
         </is>
       </c>
       <c r="D44" s="14" t="n">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="E44" s="14" t="n">
-        <v>46131</v>
+        <v>46124</v>
       </c>
       <c r="F44" s="15" t="n">
         <v>1</v>
@@ -4214,15 +4329,15 @@
       <c r="O44" s="18" t="n"/>
       <c r="P44" s="17" t="n"/>
       <c r="Q44" s="17" t="n"/>
-      <c r="R44" s="17" t="n"/>
-      <c r="S44" s="22" t="n"/>
+      <c r="R44" s="21" t="n"/>
+      <c r="S44" s="17" t="n"/>
       <c r="T44" s="17" t="n"/>
       <c r="U44" s="17" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Admin Dashboard Charts (recharts/chart.js)</t>
+          <t>Invoice Module UI (view/download PDF)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -4232,17 +4347,17 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 6</t>
         </is>
       </c>
       <c r="D45" s="14" t="n">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="E45" s="14" t="n">
         <v>46131</v>
       </c>
       <c r="F45" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" s="17" t="n"/>
       <c r="H45" s="17" t="n"/>
@@ -4255,35 +4370,35 @@
       <c r="O45" s="18" t="n"/>
       <c r="P45" s="17" t="n"/>
       <c r="Q45" s="17" t="n"/>
-      <c r="R45" s="22" t="n"/>
-      <c r="S45" s="22" t="n"/>
+      <c r="R45" s="17" t="n"/>
+      <c r="S45" s="21" t="n"/>
       <c r="T45" s="17" t="n"/>
       <c r="U45" s="17" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Reporting APIs (sales, top products, analytics)</t>
+          <t>Admin Dashboard Charts (recharts/chart.js)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D46" s="14" t="n">
         <v>46118</v>
       </c>
       <c r="E46" s="14" t="n">
-        <v>46124</v>
+        <v>46131</v>
       </c>
       <c r="F46" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="17" t="n"/>
       <c r="H46" s="17" t="n"/>
@@ -4296,35 +4411,35 @@
       <c r="O46" s="18" t="n"/>
       <c r="P46" s="17" t="n"/>
       <c r="Q46" s="17" t="n"/>
-      <c r="R46" s="22" t="n"/>
-      <c r="S46" s="17" t="n"/>
+      <c r="R46" s="21" t="n"/>
+      <c r="S46" s="21" t="n"/>
       <c r="T46" s="17" t="n"/>
       <c r="U46" s="17" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking Backend + UI</t>
+          <t>Reporting APIs (sales, top products, analytics)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Dev 7</t>
+          <t>Dev 3</t>
         </is>
       </c>
       <c r="D47" s="14" t="n">
         <v>46118</v>
       </c>
       <c r="E47" s="14" t="n">
-        <v>46131</v>
+        <v>46124</v>
       </c>
       <c r="F47" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" s="17" t="n"/>
       <c r="H47" s="17" t="n"/>
@@ -4337,35 +4452,35 @@
       <c r="O47" s="18" t="n"/>
       <c r="P47" s="17" t="n"/>
       <c r="Q47" s="17" t="n"/>
-      <c r="R47" s="22" t="n"/>
-      <c r="S47" s="22" t="n"/>
+      <c r="R47" s="21" t="n"/>
+      <c r="S47" s="17" t="n"/>
       <c r="T47" s="17" t="n"/>
       <c r="U47" s="17" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Notifications Backend (Email/SMS)</t>
+          <t>Delivery Tracking Backend + UI</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Dev 4</t>
+          <t>Dev 7</t>
         </is>
       </c>
       <c r="D48" s="14" t="n">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="E48" s="14" t="n">
         <v>46131</v>
       </c>
       <c r="F48" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="17" t="n"/>
       <c r="H48" s="17" t="n"/>
@@ -4378,83 +4493,83 @@
       <c r="O48" s="18" t="n"/>
       <c r="P48" s="17" t="n"/>
       <c r="Q48" s="17" t="n"/>
-      <c r="R48" s="17" t="n"/>
-      <c r="S48" s="22" t="n"/>
+      <c r="R48" s="21" t="n"/>
+      <c r="S48" s="21" t="n"/>
       <c r="T48" s="17" t="n"/>
       <c r="U48" s="17" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Notifications Backend (Email/SMS)</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="n">
+        <v>46125</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>46131</v>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="17" t="n"/>
+      <c r="H49" s="17" t="n"/>
+      <c r="I49" s="17" t="n"/>
+      <c r="J49" s="17" t="n"/>
+      <c r="K49" s="17" t="n"/>
+      <c r="L49" s="17" t="n"/>
+      <c r="M49" s="17" t="n"/>
+      <c r="N49" s="17" t="n"/>
+      <c r="O49" s="18" t="n"/>
+      <c r="P49" s="17" t="n"/>
+      <c r="Q49" s="17" t="n"/>
+      <c r="R49" s="17" t="n"/>
+      <c r="S49" s="21" t="n"/>
+      <c r="T49" s="17" t="n"/>
+      <c r="U49" s="17" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>PHASE 4: POLISH &amp; LAUNCH (Apr 21 - Apr 30) 🚀 DEADLINE</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="5" t="n"/>
-      <c r="I49" s="5" t="n"/>
-      <c r="J49" s="5" t="n"/>
-      <c r="K49" s="5" t="n"/>
-      <c r="L49" s="5" t="n"/>
-      <c r="M49" s="5" t="n"/>
-      <c r="N49" s="5" t="n"/>
-      <c r="O49" s="5" t="n"/>
-      <c r="P49" s="5" t="n"/>
-      <c r="Q49" s="5" t="n"/>
-      <c r="R49" s="5" t="n"/>
-      <c r="S49" s="5" t="n"/>
-      <c r="T49" s="5" t="n"/>
-      <c r="U49" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>Dev 1, Dev 6</t>
-        </is>
-      </c>
-      <c r="D50" s="14" t="n">
-        <v>46132</v>
-      </c>
-      <c r="E50" s="14" t="n">
-        <v>46138</v>
-      </c>
-      <c r="F50" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" s="17" t="n"/>
-      <c r="H50" s="17" t="n"/>
-      <c r="I50" s="17" t="n"/>
-      <c r="J50" s="17" t="n"/>
-      <c r="K50" s="17" t="n"/>
-      <c r="L50" s="17" t="n"/>
-      <c r="M50" s="17" t="n"/>
-      <c r="N50" s="17" t="n"/>
-      <c r="O50" s="18" t="n"/>
-      <c r="P50" s="17" t="n"/>
-      <c r="Q50" s="17" t="n"/>
-      <c r="R50" s="17" t="n"/>
-      <c r="S50" s="17" t="n"/>
-      <c r="T50" s="23" t="n"/>
-      <c r="U50" s="17" t="n"/>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="5" t="n"/>
+      <c r="I50" s="5" t="n"/>
+      <c r="J50" s="5" t="n"/>
+      <c r="K50" s="5" t="n"/>
+      <c r="L50" s="5" t="n"/>
+      <c r="M50" s="5" t="n"/>
+      <c r="N50" s="5" t="n"/>
+      <c r="O50" s="5" t="n"/>
+      <c r="P50" s="5" t="n"/>
+      <c r="Q50" s="5" t="n"/>
+      <c r="R50" s="5" t="n"/>
+      <c r="S50" s="5" t="n"/>
+      <c r="T50" s="5" t="n"/>
+      <c r="U50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Reporting Dashboard Charts (frontend)</t>
+          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -4464,7 +4579,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 1, Dev 6</t>
         </is>
       </c>
       <c r="D51" s="14" t="n">
@@ -4489,13 +4604,13 @@
       <c r="Q51" s="17" t="n"/>
       <c r="R51" s="17" t="n"/>
       <c r="S51" s="17" t="n"/>
-      <c r="T51" s="23" t="n"/>
+      <c r="T51" s="22" t="n"/>
       <c r="U51" s="17" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>Responsive Design + Mobile Polish</t>
+          <t>Reporting Dashboard Charts (frontend)</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -4505,7 +4620,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D52" s="14" t="n">
@@ -4530,23 +4645,23 @@
       <c r="Q52" s="17" t="n"/>
       <c r="R52" s="17" t="n"/>
       <c r="S52" s="17" t="n"/>
-      <c r="T52" s="23" t="n"/>
+      <c r="T52" s="22" t="n"/>
       <c r="U52" s="17" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Integration Testing (API + UI)</t>
+          <t>Responsive Design + Mobile Polish</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>All Devs</t>
+          <t>Dev 3</t>
         </is>
       </c>
       <c r="D53" s="14" t="n">
@@ -4571,13 +4686,13 @@
       <c r="Q53" s="17" t="n"/>
       <c r="R53" s="17" t="n"/>
       <c r="S53" s="17" t="n"/>
-      <c r="T53" s="23" t="n"/>
+      <c r="T53" s="22" t="n"/>
       <c r="U53" s="17" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>Bug Fixes &amp; Performance Optimization</t>
+          <t>Integration Testing (API + UI)</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -4591,10 +4706,10 @@
         </is>
       </c>
       <c r="D54" s="14" t="n">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="E54" s="14" t="n">
-        <v>46145</v>
+        <v>46138</v>
       </c>
       <c r="F54" s="15" t="n">
         <v>1</v>
@@ -4612,13 +4727,13 @@
       <c r="Q54" s="17" t="n"/>
       <c r="R54" s="17" t="n"/>
       <c r="S54" s="17" t="n"/>
-      <c r="T54" s="17" t="n"/>
-      <c r="U54" s="23" t="n"/>
+      <c r="T54" s="22" t="n"/>
+      <c r="U54" s="17" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>UAT + Production Deployment</t>
+          <t>Bug Fixes &amp; Performance Optimization</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -4654,111 +4769,151 @@
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="17" t="n"/>
       <c r="T55" s="17" t="n"/>
-      <c r="U55" s="23" t="n"/>
+      <c r="U55" s="22" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="24" t="inlineStr">
-        <is>
-          <t>▲ TODAY (Mar 16, 2026) — 6.4 weeks to deadline</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="n"/>
-      <c r="C56" s="25" t="n"/>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="25" t="n"/>
-      <c r="F56" s="25" t="n"/>
-      <c r="G56" s="25" t="n"/>
-      <c r="H56" s="25" t="n"/>
-      <c r="I56" s="25" t="n"/>
-      <c r="J56" s="25" t="n"/>
-      <c r="K56" s="25" t="n"/>
-      <c r="L56" s="25" t="n"/>
-      <c r="M56" s="25" t="n"/>
-      <c r="N56" s="25" t="n"/>
-      <c r="O56" s="26" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>UAT + Production Deployment</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Full Stack</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>All Devs</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E56" s="14" t="n">
+        <v>46145</v>
+      </c>
+      <c r="F56" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="17" t="n"/>
+      <c r="J56" s="17" t="n"/>
+      <c r="K56" s="17" t="n"/>
+      <c r="L56" s="17" t="n"/>
+      <c r="M56" s="17" t="n"/>
+      <c r="N56" s="17" t="n"/>
+      <c r="O56" s="18" t="n"/>
+      <c r="P56" s="17" t="n"/>
+      <c r="Q56" s="17" t="n"/>
+      <c r="R56" s="17" t="n"/>
+      <c r="S56" s="17" t="n"/>
+      <c r="T56" s="17" t="n"/>
+      <c r="U56" s="22" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>▲ TODAY (Mar 21, 2026) — 5.7 weeks to deadline</t>
+        </is>
+      </c>
+      <c r="B57" s="24" t="n"/>
+      <c r="C57" s="24" t="n"/>
+      <c r="D57" s="24" t="n"/>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="24" t="n"/>
+      <c r="G57" s="24" t="n"/>
+      <c r="H57" s="24" t="n"/>
+      <c r="I57" s="24" t="n"/>
+      <c r="J57" s="24" t="n"/>
+      <c r="K57" s="24" t="n"/>
+      <c r="L57" s="24" t="n"/>
+      <c r="M57" s="24" t="n"/>
+      <c r="N57" s="24" t="n"/>
+      <c r="O57" s="25" t="inlineStr">
         <is>
           <t>▲ NOW</t>
         </is>
       </c>
-      <c r="P56" s="25" t="n"/>
-      <c r="Q56" s="25" t="n"/>
-      <c r="R56" s="25" t="n"/>
-      <c r="S56" s="25" t="n"/>
-      <c r="T56" s="25" t="n"/>
-      <c r="U56" s="25" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="27" t="inlineStr">
+      <c r="P57" s="24" t="n"/>
+      <c r="Q57" s="24" t="n"/>
+      <c r="R57" s="24" t="n"/>
+      <c r="S57" s="24" t="n"/>
+      <c r="T57" s="24" t="n"/>
+      <c r="U57" s="24" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
         <is>
           <t>LEGEND:</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="28" t="n"/>
-      <c r="B59" s="29" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="27" t="n"/>
+      <c r="B60" s="28" t="inlineStr">
         <is>
           <t>Completed (Jan 22 - Mar 10)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="30" t="n"/>
-      <c r="B60" s="29" t="inlineStr">
-        <is>
-          <t>Phase 1: Foundation (Mar 10-23) — mostly DONE</t>
-        </is>
-      </c>
-    </row>
     <row r="61">
-      <c r="A61" s="31" t="n"/>
-      <c r="B61" s="29" t="inlineStr">
-        <is>
-          <t>Phase 2: Core CRUD (Mar 24 - Apr 6) — frontend DONE, backend partial</t>
+      <c r="A61" s="29" t="n"/>
+      <c r="B61" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1: Foundation (Mar 10-23) — 100% DONE</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="32" t="n"/>
-      <c r="B62" s="29" t="inlineStr">
+      <c r="A62" s="30" t="n"/>
+      <c r="B62" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2: Core CRUD (Mar 24 - Apr 6) — frontend DONE, backend: Razorpay/Invoice/Pricing pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="31" t="n"/>
+      <c r="B63" s="28" t="inlineStr">
         <is>
           <t>Phase 3: Business Logic &amp; Dashboard (Apr 7-20)</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="33" t="n"/>
-      <c r="B63" s="29" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="32" t="n"/>
+      <c r="B64" s="28" t="inlineStr">
         <is>
           <t>Phase 4: Polish &amp; Launch (Apr 21-30)</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="34" t="n"/>
-      <c r="B64" s="29" t="inlineStr">
-        <is>
-          <t>TODAY marker (Mar 16)</t>
+    <row r="65">
+      <c r="A65" s="33" t="n"/>
+      <c r="B65" s="28" t="inlineStr">
+        <is>
+          <t>TODAY marker (Mar 21)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A50:U50"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="B63:D63"/>
     <mergeCell ref="B61:D61"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A41:U41"/>
-    <mergeCell ref="A49:U49"/>
     <mergeCell ref="A5:U5"/>
-    <mergeCell ref="A28:U28"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A42:U42"/>
+    <mergeCell ref="B65:D65"/>
     <mergeCell ref="A14:U14"/>
     <mergeCell ref="B62:D62"/>
-    <mergeCell ref="A23:U23"/>
+    <mergeCell ref="A27:U27"/>
     <mergeCell ref="B64:D64"/>
+    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4770,7 +4925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4779,7 +4934,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>PROJECT SUMMARY</t>
         </is>
@@ -4788,23 +4943,23 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Start: 22 Jan 2026  |  Today: 16 Mar 2026  |  Deadline: 30 Apr 2026</t>
+          <t>Start: 22 Jan 2026  |  Today: 21 Mar 2026  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr"/>
-      <c r="B4" s="36" t="inlineStr"/>
-      <c r="C4" s="36" t="inlineStr"/>
+      <c r="A4" s="35" t="inlineStr"/>
+      <c r="B4" s="35" t="inlineStr"/>
+      <c r="C4" s="35" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>TIMELINE</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr"/>
-      <c r="C5" s="37" t="inlineStr"/>
+      <c r="B5" s="36" t="inlineStr"/>
+      <c r="C5" s="36" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -4827,7 +4982,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>16 Mar 2026</t>
+          <t>21 Mar 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -4849,7 +5004,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>6.4 weeks remaining</t>
+          <t>5.7 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -4866,27 +5021,27 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>No buffer for delays</t>
+          <t>~1 week buffer if on track</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr"/>
-      <c r="B10" s="36" t="inlineStr"/>
-      <c r="C10" s="36" t="inlineStr"/>
+      <c r="A10" s="35" t="inlineStr"/>
+      <c r="B10" s="35" t="inlineStr"/>
+      <c r="C10" s="35" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>COMPLETION STATUS</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C11" s="37" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -4900,12 +5055,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>17 modules</t>
+          <t>21 modules</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Auth, Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Cart, Wishlist, Coupon, Address, Schema, Seed, Validation, RBAC</t>
+          <t>Auth, Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Cart, Wishlist, Coupon, Admin Users, Address, Schema, Seed, Validation, RBAC, Pagination, File Upload, Order State Machine, Inventory</t>
         </is>
       </c>
     </row>
@@ -4917,12 +5072,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>7 features</t>
+          <t>4 features</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Pagination, File Upload, Payments, Invoices, Reporting, Notifications, Pricing Tiers</t>
+          <t>Payments (Razorpay), Invoices (PDF), Reporting/Analytics APIs, Notifications (Email/SMS)</t>
         </is>
       </c>
     </row>
@@ -4934,12 +5089,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>3 features</t>
+          <t>2 features</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Order Workflow (needs transition validation), Inventory (needs decrement), Delivery Tracking</t>
+          <t>Pricing Tiers (coupon exists, tier logic pending), Delivery Tracking (basic fields, no logistics API)</t>
         </is>
       </c>
     </row>
@@ -4951,12 +5106,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>48 items</t>
+          <t>54 items</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>All admin CRUD (9 modules), all storefront pages (11), buyer account (4), foundation (10), UI components (4), nav/footer</t>
+          <t>All admin CRUD (11 modules incl. Coupons &amp; Admin Users), all storefront pages (11), buyer account (4), foundation (10), UI components (4), file upload UI, nav/footer</t>
         </is>
       </c>
     </row>
@@ -4968,50 +5123,50 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>8 items</t>
+          <t>7 items</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Inventory UI, Payment UI, Invoice UI, Delivery UI, Dashboard Charts, Role-based Dashboards, File Upload UI, Responsive polish</t>
+          <t>Inventory UI, Payment UI, Invoice UI, Delivery UI, Dashboard Charts, Role-based Dashboards, Responsive polish</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="inlineStr"/>
-      <c r="B17" s="36" t="inlineStr"/>
-      <c r="C17" s="36" t="inlineStr"/>
+      <c r="A17" s="35" t="inlineStr"/>
+      <c r="B17" s="35" t="inlineStr"/>
+      <c r="C17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>Overall Completion</t>
         </is>
       </c>
-      <c r="B18" s="38" t="inlineStr">
-        <is>
-          <t>~60%</t>
-        </is>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>Backend CRUD + Frontend CRUD + Storefront all done. Remaining: business logic backends + specialized UIs.</t>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>~70%</t>
+        </is>
+      </c>
+      <c r="C18" s="38" t="inlineStr">
+        <is>
+          <t>Phase 1 100% done. Phase 2 frontend done. Remaining: 4 backend features + 7 frontend UIs + testing/deployment.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="inlineStr"/>
-      <c r="B19" s="36" t="inlineStr"/>
-      <c r="C19" s="36" t="inlineStr"/>
+      <c r="A19" s="35" t="inlineStr"/>
+      <c r="B19" s="35" t="inlineStr"/>
+      <c r="C19" s="35" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="37" t="inlineStr">
+      <c r="A20" s="36" t="inlineStr">
         <is>
           <t>RISK ASSESSMENT</t>
         </is>
       </c>
-      <c r="B20" s="37" t="inlineStr"/>
-      <c r="C20" s="37" t="inlineStr"/>
+      <c r="B20" s="36" t="inlineStr"/>
+      <c r="C20" s="36" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -5019,14 +5174,14 @@
           <t>Schedule Risk</t>
         </is>
       </c>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>LOW-MEDIUM</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Ahead of schedule on frontend. ~40% work in 6.4 weeks. Manageable with focus.</t>
+          <t>Ahead of schedule. Phase 1 fully done. ~30% work in 5.7 weeks. Comfortable pace.</t>
         </is>
       </c>
     </row>
@@ -5038,12 +5193,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Payments + Invoices + Inventory</t>
+          <t>Razorpay + Invoice PDF</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>These depend on each other — must start this week</t>
+          <t>Payment backend needed before Payment UI; Invoice backend needed before Invoice UI</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5215,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Backend features (pagination, upload, payments) + Frontend UIs simultaneously</t>
+          <t>Backend (Razorpay, Invoice, Reporting) + Frontend (Inventory UI, Charts) simultaneously</t>
         </is>
       </c>
     </row>
@@ -5072,32 +5227,32 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>FOCUSED SPRINTS</t>
+          <t>START PHASE 2 BACKEND</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Tackle P0 items (pagination, upload, state machine, inventory) this week</t>
+          <t>Begin Razorpay integration and Invoice PDF generation next week</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="36" t="inlineStr"/>
-      <c r="B25" s="36" t="inlineStr"/>
-      <c r="C25" s="36" t="inlineStr"/>
+      <c r="A25" s="35" t="inlineStr"/>
+      <c r="B25" s="35" t="inlineStr"/>
+      <c r="C25" s="35" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="37" t="inlineStr">
+      <c r="A26" s="36" t="inlineStr">
         <is>
           <t>PHASE PLAN (REMAINING)</t>
         </is>
       </c>
-      <c r="B26" s="37" t="inlineStr">
+      <c r="B26" s="36" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C26" s="36" t="inlineStr">
         <is>
           <t>Focus</t>
         </is>
@@ -5106,17 +5261,17 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Phase 1 Remaining</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Mar 16-23 (1 wk)</t>
+          <t>COMPLETED ✅</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Pagination, File Upload, Order State Machine, Inventory Decrement</t>
+          <t>All items done: Pagination, File Upload, Order State Machine, Inventory Decrement</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5288,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation, Product file upload UI</t>
+          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation</t>
         </is>
       </c>
     </row>
@@ -5172,23 +5327,23 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="36" t="inlineStr"/>
-      <c r="B31" s="36" t="inlineStr"/>
-      <c r="C31" s="36" t="inlineStr"/>
+      <c r="A31" s="35" t="inlineStr"/>
+      <c r="B31" s="35" t="inlineStr"/>
+      <c r="C31" s="35" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="37" t="inlineStr">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>WHAT WAS DONE AHEAD OF SCHEDULE</t>
         </is>
       </c>
-      <c r="B32" s="37" t="inlineStr"/>
-      <c r="C32" s="37" t="inlineStr"/>
+      <c r="B32" s="36" t="inlineStr"/>
+      <c r="C32" s="36" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>All Admin CRUD UIs (9 modules)</t>
+          <t>All Admin CRUD UIs (11 modules)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -5198,7 +5353,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard</t>
+          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard, Coupons, Admin Users</t>
         </is>
       </c>
     </row>
@@ -5254,107 +5409,141 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="36" t="inlineStr"/>
-      <c r="B37" s="36" t="inlineStr"/>
-      <c r="C37" s="36" t="inlineStr"/>
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Phase 1 Backend (4 items)</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Done on time (Mar 17)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Pagination, Multer upload, Order state machine, Inventory decrement</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="37" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Coupons + Admin Users (legacy admin)</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Done Mar 21</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Full CRUD modules added to both React frontend and legacy admin panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr"/>
+      <c r="B39" s="35" t="inlineStr"/>
+      <c r="C39" s="35" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="36" t="inlineStr">
         <is>
           <t>TEAM ALLOCATION (suggested for remaining)</t>
         </is>
       </c>
-      <c r="B38" s="37" t="inlineStr"/>
-      <c r="C38" s="37" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Dev 1 (Frontend Lead)</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>File Upload UI → Role-based Dashboards → Responsive polish</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Dev 2 (Frontend)</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr"/>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>Dashboard Charts → Reporting UI → Integration testing</t>
-        </is>
-      </c>
+      <c r="B40" s="36" t="inlineStr"/>
+      <c r="C40" s="36" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Dev 3 (Backend + Frontend)</t>
+          <t>Dev 1 (Frontend Lead)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr"/>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Pagination → Invoice PDF backend → Reporting APIs</t>
+          <t>Inventory UI → Role-based Dashboards → Responsive polish</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Dev 4 (Backend Lead)</t>
+          <t>Dev 2 (Frontend)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr"/>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>File Upload Multer → Inventory decrement → Notifications</t>
+          <t>Dashboard Charts → Reporting UI → Integration testing</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Dev 5 (Frontend)</t>
+          <t>Dev 3 (Backend + Frontend)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Inventory UI → Dashboard charts → Responsive design</t>
+          <t>Invoice PDF backend → Reporting APIs → Invoice UI</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Dev 6 (Frontend)</t>
+          <t>Dev 4 (Backend Lead)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr"/>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Payment UI → Invoice UI → Role-based views</t>
+          <t>Pricing Tiers → Notifications (Email/SMS)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Dev 7 (Backend)</t>
+          <t>Dev 5 (Frontend)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr"/>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Order State Machine → Razorpay → Delivery tracking</t>
+          <t>Dashboard Charts → Responsive design</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Dev 6 (Frontend)</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Payment UI → Invoice UI → Role-based views</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Dev 7 (Backend)</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Razorpay integration → Delivery tracking backend + UI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Gantt chart: refresh all statuses to Mar 23, 2026
- Updated today marker from Mar 21 → Mar 23
- Added completed items: back-order logic, auto-entity creation,
  logo branding, token auto-refresh, deployment guide, work report
- Backend completed count: 21 → 24 modules
- Frontend completed count: 54 → 57 items
- Overall completion: ~70% → ~72%
- Updated remaining weeks calculation (5.4 weeks to deadline)

https://claude.ai/code/session_0147TWQhvrJuRoRZiqK4BvoS
</commit_message>
<xml_diff>
--- a/MaterialKing_Gantt_Chart.xlsx
+++ b/MaterialKing_Gantt_Chart.xlsx
@@ -649,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 21 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  5.7 weeks remaining</t>
+          <t>Generated: 23 Mar 2026  |  Team: 6-7 devs  |  Start: 22 Jan 2026  |  Deadline: 30 Apr 2026  |  5.4 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>BACKEND - COMPLETED (Jan 22 - Mar 21)</t>
+          <t>BACKEND - COMPLETED (Jan 22 - Mar 23)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -1167,24 +1167,36 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - FOUNDATION (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Back-order Logic (never reject on low stock)</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Accept all orders; mark items as back-order with 15-20 day timeline — completed Mar 21</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Vite + React 19 + TypeScript</t>
+          <t>Auto-create Buyer/Vendor/Dealer on Registration</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1194,19 +1206,19 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Project scaffolded and running</t>
+          <t>Insert entity record during user registration + backfill script — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Tailwind CSS Config (custom MK theme)</t>
+          <t>Bug Fixes (auth, coupon, token refresh)</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -1216,36 +1228,24 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>mk-red, mk-gray palette, Montserrat font</t>
+          <t>Fixed duplicate phone key, coupon integer parse, 401 token refresh — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>BrowserRouter + Route Definitions</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Full route tree: public, admin, account sections</t>
-        </is>
-      </c>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - FOUNDATION (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>React Query (QueryClientProvider)</t>
+          <t>Vite + React 19 + TypeScript</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -1260,14 +1260,14 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Configured with retry:1, staleTime:30s</t>
+          <t>Project scaffolded and running</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Axios API Client + Token Refresh</t>
+          <t>Tailwind CSS Config (custom MK theme)</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1282,14 +1282,14 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Auto-refresh on 401, concurrent request queue</t>
+          <t>mk-red, mk-gray palette, Montserrat font</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AuthContext + useAuth hook</t>
+          <t>BrowserRouter + Route Definitions</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -1304,14 +1304,14 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Login/logout/updateUser/isAdmin, auto-load on mount</t>
+          <t>Full route tree: public, admin, account sections</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Protected Routes / Route Guards</t>
+          <t>React Query (QueryClientProvider)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>ProtectedRoute component with loading spinner</t>
+          <t>Configured with retry:1, staleTime:30s</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>API Service Layer (13 modules)</t>
+          <t>Axios API Client + Token Refresh</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1348,14 +1348,14 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>product, category, brand, vendor, zone, dealer, buyer, order, auth, cart, coupon, wishlist, address, adminUser</t>
+          <t>Auto-refresh on 401, concurrent request queue</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Login Page</t>
+          <t>AuthContext + useAuth hook</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1370,14 +1370,14 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Email/password login with validation</t>
+          <t>Login/logout/updateUser/isAdmin, auto-load on mount</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Register Page</t>
+          <t>Protected Routes / Route Guards</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1392,24 +1392,36 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>User registration with role selection</t>
+          <t>ProtectedRoute component with loading spinner</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - ADMIN CRUD MODULES (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>API Service Layer (13 modules)</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>product, category, brand, vendor, zone, dealer, buyer, order, auth, cart, coupon, wishlist, address, adminUser</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Admin Dashboard</t>
+          <t>Login Page</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1424,14 +1436,14 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Stats cards (orders, revenue, products, buyers, dealers) + recent orders table</t>
+          <t>Email/password login with validation</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Products Module (list + forms)</t>
+          <t>Register Page</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -1446,36 +1458,24 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Full CRUD with 4-tab form (basic, dimensions, attributes, packaging)</t>
+          <t>User registration with role selection</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Brands Module (list + forms)</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>CRUD with DataTable + FormModal</t>
-        </is>
-      </c>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - ADMIN CRUD MODULES (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Categories Module (list + forms)</t>
+          <t>Admin Dashboard</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -1490,14 +1490,14 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>CRUD with parent/child hierarchy</t>
+          <t>Stats cards (orders, revenue, products, buyers, dealers) + recent orders table</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Vendors Module (list + forms)</t>
+          <t>Products Module (list + forms)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -1512,14 +1512,14 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>CRUD with DataTable + FormModal</t>
+          <t>Full CRUD with 4-tab form (basic, dimensions, attributes, packaging)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Zones Module (list + forms)</t>
+          <t>Brands Module (list + forms)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Buyers Module (list + forms)</t>
+          <t>Categories Module (list + forms)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -1556,14 +1556,14 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>CRUD with DataTable + FormModal</t>
+          <t>CRUD with parent/child hierarchy</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Dealers Module (list + forms)</t>
+          <t>Vendors Module (list + forms)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Orders Module (list + detail)</t>
+          <t>Zones Module (list + forms)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -1600,14 +1600,14 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Admin order management with status updates</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Coupons Module (list + forms)</t>
+          <t>Buyers Module (list + forms)</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -1622,14 +1622,14 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Admin Users Module (list + forms)</t>
+          <t>Dealers Module (list + forms)</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -1644,14 +1644,14 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
+          <t>CRUD with DataTable + FormModal</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Reusable UI Components</t>
+          <t>Orders Module (list + detail)</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -1666,14 +1666,14 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>DataTable, FormField, FormModal, StatusBadge</t>
+          <t>Admin order management with status updates</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Products File Upload UI</t>
+          <t>Coupons Module (list + forms)</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -1688,24 +1688,36 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Tech Data Sheet PDF upload in product forms — completed Mar 17</t>
+          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - STOREFRONT PAGES (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Admin Users Module (list + forms)</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Full CRUD in both React frontend and legacy admin panel — completed Mar 21</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Public Header + Nav with Category Hover Dropdowns</t>
+          <t>Reusable UI Components</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -1720,14 +1732,14 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>7 merged categories, hover subcategory menus, linked to products</t>
+          <t>DataTable, FormField, FormModal, StatusBadge</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>Public Footer</t>
+          <t>Products File Upload UI</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -1742,14 +1754,14 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Footer with correct office address</t>
+          <t>Tech Data Sheet PDF upload in product forms — completed Mar 17</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Home Page</t>
+          <t>Material King Logo &amp; Branding</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -1764,14 +1776,14 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Hero section + featured products</t>
+          <t>Logo added to all 3 frontends (storefront, admin, legacy admin) — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>Products List Page</t>
+          <t>Token Auto-Refresh (Admin Panel)</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -1786,36 +1798,24 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Filters (category, brand, price range, search, sort)</t>
+          <t>401 interceptor with automatic token refresh — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>Product Detail Page</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Product info tabs, wishlist, add to cart</t>
-        </is>
-      </c>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - STOREFRONT PAGES (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>Categories Page</t>
+          <t>Public Header + Nav with Category Hover Dropdowns</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -1830,14 +1830,14 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Category grid with subcategory tags</t>
+          <t>7 merged categories, hover subcategory menus, linked to products</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Cart Page</t>
+          <t>Public Footer</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -1852,14 +1852,14 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Cart items, coupon apply, tax/shipping calc</t>
+          <t>Footer with correct office address</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Checkout Page</t>
+          <t>Home Page</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -1874,14 +1874,14 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Address selection, payment method, order placement</t>
+          <t>Hero section + featured products</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>Order Confirmation Page</t>
+          <t>Products List Page</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -1896,14 +1896,14 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Post-checkout confirmation (protected)</t>
+          <t>Filters (category, brand, price range, search, sort)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>About Page</t>
+          <t>Product Detail Page</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -1918,14 +1918,14 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Static about us page</t>
+          <t>Product info tabs, wishlist, add to cart</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>Contact Page</t>
+          <t>Categories Page</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -1940,24 +1940,36 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Contact form with office address</t>
+          <t>Category grid with subcategory tags</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - BUYER ACCOUNT (COMPLETED)</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="5" t="n"/>
-      <c r="D64" s="5" t="n"/>
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Cart Page</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>Cart items, coupon apply, tax/shipping calc</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>My Account Page</t>
+          <t>Checkout Page</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -1972,14 +1984,14 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Profile management</t>
+          <t>Address selection, payment method, order placement</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>My Orders Page</t>
+          <t>Order Confirmation Page</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -1994,14 +2006,14 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Order history with detail view</t>
+          <t>Post-checkout confirmation (protected)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Addresses Page</t>
+          <t>About Page</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -2016,14 +2028,14 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Saved addresses CRUD with default</t>
+          <t>Static about us page</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Wishlist Page</t>
+          <t>Contact Page</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -2038,14 +2050,14 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Wishlist management</t>
+          <t>Contact form with office address</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>BACKEND - PENDING (must complete by Apr 30)</t>
+          <t>FRONTEND - BUYER ACCOUNT (COMPLETED)</t>
         </is>
       </c>
       <c r="B69" s="5" t="n"/>
@@ -2055,198 +2067,186 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>Payment Integration (Razorpay)</t>
+          <t>My Account Page</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>No payment gateway code. Only COD supported</t>
+          <t>Profile management</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Invoice Generation (PDF)</t>
+          <t>My Orders Page</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>No PDF generation library or templates</t>
+          <t>Order history with detail view</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>Pricing Tiers / Discount Structures</t>
+          <t>Addresses Page</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
+          <t>Saved addresses CRUD with default</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking</t>
+          <t>Wishlist Page</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Basic date fields; no tracking numbers or logistics API</t>
+          <t>Wishlist management</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>Reporting / Analytics APIs</t>
-        </is>
-      </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>No sales reports, trend analytics, export APIs</t>
-        </is>
-      </c>
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>DOCUMENTATION (COMPLETED)</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Notifications (Email/SMS)</t>
+          <t>Deployment Guide (Ubuntu, Node, PG, Nginx, SSL, PM2)</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>No nodemailer/twilio integration</t>
+          <t>Full production deployment docs with SQL backup/restore — completed Mar 21</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>FRONTEND - PENDING (must complete by Apr 30)</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="n"/>
-      <c r="C76" s="5" t="n"/>
-      <c r="D76" s="5" t="n"/>
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Daily Work Report (Mar 21)</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Comprehensive testing report for all frontend/backend/admin modules</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>Inventory Module UI</t>
+          <t>Gantt Chart Updates</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Stock levels, alerts, reorder points dashboard</t>
+          <t>Refreshed to Mar 23, 2026 with all completed items</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>Payment Module UI</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>Payment processing screens (Razorpay integration)</t>
-        </is>
-      </c>
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>BACKEND - PENDING (must complete by Apr 30)</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Invoice Module UI</t>
+          <t>Payment Integration (Razorpay)</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -2256,19 +2256,19 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>View/download invoices as PDF</t>
+          <t>No payment gateway code. Only COD supported</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking UI</t>
+          <t>Invoice Generation (PDF)</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
@@ -2278,109 +2278,296 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Track order delivery status with timeline</t>
+          <t>No PDF generation library or templates</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>Reporting / Dashboard Charts</t>
+          <t>Pricing Tiers / Discount Structures</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Sales summary, top products, dealer analytics with charts</t>
+          <t>Dealer credit + coupon system exists; tier-based pricing logic not implemented</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+          <t>Delivery Tracking</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>Different dashboards per role</t>
+          <t>Basic date fields; no tracking numbers or logistics API</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>Responsive Design / Mobile</t>
+          <t>Reporting / Analytics APIs</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C83" s="9" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Desktop works; mobile nav exists but needs polish</t>
+          <t>No sales reports, trend analytics, export APIs</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
+          <t>Notifications (Email/SMS)</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>No nodemailer/twilio integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>FRONTEND - PENDING (must complete by Apr 30)</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n"/>
+      <c r="C85" s="5" t="n"/>
+      <c r="D85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>Inventory Module UI</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Stock levels, alerts, reorder points dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>Payment Module UI</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>Payment processing screens (Razorpay integration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Invoice Module UI</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>View/download invoices as PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>Delivery Tracking UI</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>Track order delivery status with timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>Reporting / Dashboard Charts</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>Sales summary, top products, dealer analytics with charts</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>Different dashboards per role</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>Responsive Design / Mobile</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>Desktop works; mobile nav exists but needs polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
           <t>Admin Dashboard Charts</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C84" s="9" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr">
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>Stats cards done; no charts/graphs, no date-range analytics</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A74:D74"/>
     <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A41:D41"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A85:D85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2392,7 +2579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U65"/>
+  <dimension ref="A1:U68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2428,7 +2615,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 8 weeks  |  REMAINING: 5.7 weeks  |  Deadline: 30 Apr 2026</t>
+          <t>Team: 6-7 Developers  |  Total: 14 Weeks  |  Elapsed: 9 weeks  |  REMAINING: 5.4 weeks  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -2511,13 +2698,13 @@
 09 Mar</t>
         </is>
       </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="O4" s="11" t="inlineStr">
         <is>
           <t>W9
 16 Mar</t>
         </is>
       </c>
-      <c r="P4" s="11" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>W10
 23 Mar</t>
@@ -2622,8 +2809,8 @@
       <c r="L6" s="17" t="n"/>
       <c r="M6" s="17" t="n"/>
       <c r="N6" s="17" t="n"/>
-      <c r="O6" s="18" t="n"/>
-      <c r="P6" s="17" t="n"/>
+      <c r="O6" s="17" t="n"/>
+      <c r="P6" s="18" t="n"/>
       <c r="Q6" s="17" t="n"/>
       <c r="R6" s="17" t="n"/>
       <c r="S6" s="17" t="n"/>
@@ -2671,8 +2858,8 @@
       <c r="L7" s="17" t="n"/>
       <c r="M7" s="17" t="n"/>
       <c r="N7" s="17" t="n"/>
-      <c r="O7" s="18" t="n"/>
-      <c r="P7" s="17" t="n"/>
+      <c r="O7" s="17" t="n"/>
+      <c r="P7" s="18" t="n"/>
       <c r="Q7" s="17" t="n"/>
       <c r="R7" s="17" t="n"/>
       <c r="S7" s="17" t="n"/>
@@ -2720,8 +2907,8 @@
       <c r="L8" s="17" t="n"/>
       <c r="M8" s="17" t="n"/>
       <c r="N8" s="17" t="n"/>
-      <c r="O8" s="18" t="n"/>
-      <c r="P8" s="17" t="n"/>
+      <c r="O8" s="17" t="n"/>
+      <c r="P8" s="18" t="n"/>
       <c r="Q8" s="17" t="n"/>
       <c r="R8" s="17" t="n"/>
       <c r="S8" s="17" t="n"/>
@@ -2769,8 +2956,8 @@
       <c r="L9" s="17" t="n"/>
       <c r="M9" s="17" t="n"/>
       <c r="N9" s="17" t="n"/>
-      <c r="O9" s="18" t="n"/>
-      <c r="P9" s="17" t="n"/>
+      <c r="O9" s="17" t="n"/>
+      <c r="P9" s="18" t="n"/>
       <c r="Q9" s="17" t="n"/>
       <c r="R9" s="17" t="n"/>
       <c r="S9" s="17" t="n"/>
@@ -2822,8 +3009,8 @@
         </is>
       </c>
       <c r="N10" s="17" t="n"/>
-      <c r="O10" s="18" t="n"/>
-      <c r="P10" s="17" t="n"/>
+      <c r="O10" s="17" t="n"/>
+      <c r="P10" s="18" t="n"/>
       <c r="Q10" s="17" t="n"/>
       <c r="R10" s="17" t="n"/>
       <c r="S10" s="17" t="n"/>
@@ -2871,8 +3058,8 @@
         </is>
       </c>
       <c r="N11" s="17" t="n"/>
-      <c r="O11" s="18" t="n"/>
-      <c r="P11" s="17" t="n"/>
+      <c r="O11" s="17" t="n"/>
+      <c r="P11" s="18" t="n"/>
       <c r="Q11" s="17" t="n"/>
       <c r="R11" s="17" t="n"/>
       <c r="S11" s="17" t="n"/>
@@ -2920,8 +3107,8 @@
         </is>
       </c>
       <c r="N12" s="17" t="n"/>
-      <c r="O12" s="18" t="n"/>
-      <c r="P12" s="17" t="n"/>
+      <c r="O12" s="17" t="n"/>
+      <c r="P12" s="18" t="n"/>
       <c r="Q12" s="17" t="n"/>
       <c r="R12" s="17" t="n"/>
       <c r="S12" s="17" t="n"/>
@@ -2969,8 +3156,8 @@
         </is>
       </c>
       <c r="N13" s="17" t="n"/>
-      <c r="O13" s="18" t="n"/>
-      <c r="P13" s="17" t="n"/>
+      <c r="O13" s="17" t="n"/>
+      <c r="P13" s="18" t="n"/>
       <c r="Q13" s="17" t="n"/>
       <c r="R13" s="17" t="n"/>
       <c r="S13" s="17" t="n"/>
@@ -3041,8 +3228,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" s="18" t="n"/>
-      <c r="P15" s="17" t="n"/>
+      <c r="O15" s="17" t="n"/>
+      <c r="P15" s="18" t="n"/>
       <c r="Q15" s="17" t="n"/>
       <c r="R15" s="17" t="n"/>
       <c r="S15" s="17" t="n"/>
@@ -3086,8 +3273,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O16" s="18" t="n"/>
-      <c r="P16" s="17" t="n"/>
+      <c r="O16" s="17" t="n"/>
+      <c r="P16" s="18" t="n"/>
       <c r="Q16" s="17" t="n"/>
       <c r="R16" s="17" t="n"/>
       <c r="S16" s="17" t="n"/>
@@ -3131,8 +3318,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" s="18" t="n"/>
-      <c r="P17" s="17" t="n"/>
+      <c r="O17" s="17" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="17" t="n"/>
       <c r="R17" s="17" t="n"/>
       <c r="S17" s="17" t="n"/>
@@ -3176,8 +3363,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O18" s="18" t="n"/>
-      <c r="P18" s="17" t="n"/>
+      <c r="O18" s="17" t="n"/>
+      <c r="P18" s="18" t="n"/>
       <c r="Q18" s="17" t="n"/>
       <c r="R18" s="17" t="n"/>
       <c r="S18" s="17" t="n"/>
@@ -3221,8 +3408,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O19" s="18" t="n"/>
-      <c r="P19" s="17" t="n"/>
+      <c r="O19" s="17" t="n"/>
+      <c r="P19" s="18" t="n"/>
       <c r="Q19" s="17" t="n"/>
       <c r="R19" s="17" t="n"/>
       <c r="S19" s="17" t="n"/>
@@ -3271,7 +3458,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P20" s="17" t="n"/>
+      <c r="P20" s="18" t="n"/>
       <c r="Q20" s="17" t="n"/>
       <c r="R20" s="17" t="n"/>
       <c r="S20" s="17" t="n"/>
@@ -3320,7 +3507,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P21" s="17" t="n"/>
+      <c r="P21" s="18" t="n"/>
       <c r="Q21" s="17" t="n"/>
       <c r="R21" s="17" t="n"/>
       <c r="S21" s="17" t="n"/>
@@ -3365,7 +3552,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P22" s="17" t="n"/>
+      <c r="P22" s="18" t="n"/>
       <c r="Q22" s="17" t="n"/>
       <c r="R22" s="17" t="n"/>
       <c r="S22" s="17" t="n"/>
@@ -3410,7 +3597,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P23" s="17" t="n"/>
+      <c r="P23" s="18" t="n"/>
       <c r="Q23" s="17" t="n"/>
       <c r="R23" s="17" t="n"/>
       <c r="S23" s="17" t="n"/>
@@ -3455,7 +3642,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P24" s="17" t="n"/>
+      <c r="P24" s="18" t="n"/>
       <c r="Q24" s="17" t="n"/>
       <c r="R24" s="17" t="n"/>
       <c r="S24" s="17" t="n"/>
@@ -3500,7 +3687,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P25" s="17" t="n"/>
+      <c r="P25" s="18" t="n"/>
       <c r="Q25" s="17" t="n"/>
       <c r="R25" s="17" t="n"/>
       <c r="S25" s="17" t="n"/>
@@ -3545,7 +3732,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P26" s="17" t="n"/>
+      <c r="P26" s="18" t="n"/>
       <c r="Q26" s="17" t="n"/>
       <c r="R26" s="17" t="n"/>
       <c r="S26" s="17" t="n"/>
@@ -3553,36 +3740,54 @@
       <c r="U26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 2: CORE MODULES (Mar 24 - Apr 6) — Frontend DONE, Backend in progress</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="5" t="n"/>
-      <c r="O27" s="5" t="n"/>
-      <c r="P27" s="5" t="n"/>
-      <c r="Q27" s="5" t="n"/>
-      <c r="R27" s="5" t="n"/>
-      <c r="S27" s="5" t="n"/>
-      <c r="T27" s="5" t="n"/>
-      <c r="U27" s="5" t="n"/>
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Back-order Logic + Bug Fixes (auth, coupon, token)</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3, Dev 4</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>46097</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>46103</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="17" t="n"/>
+      <c r="H27" s="17" t="n"/>
+      <c r="I27" s="17" t="n"/>
+      <c r="J27" s="17" t="n"/>
+      <c r="K27" s="17" t="n"/>
+      <c r="L27" s="17" t="n"/>
+      <c r="M27" s="17" t="n"/>
+      <c r="N27" s="17" t="n"/>
+      <c r="O27" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P27" s="18" t="n"/>
+      <c r="Q27" s="17" t="n"/>
+      <c r="R27" s="17" t="n"/>
+      <c r="S27" s="17" t="n"/>
+      <c r="T27" s="17" t="n"/>
+      <c r="U27" s="17" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>Products Module UI (list + forms + 4 tabs)</t>
+          <t>Logo Branding (all 3 frontends)</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -3596,13 +3801,13 @@
         </is>
       </c>
       <c r="D28" s="14" t="n">
-        <v>46090</v>
+        <v>46097</v>
       </c>
       <c r="E28" s="14" t="n">
         <v>46103</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" s="17" t="n"/>
       <c r="H28" s="17" t="n"/>
@@ -3611,17 +3816,13 @@
       <c r="K28" s="17" t="n"/>
       <c r="L28" s="17" t="n"/>
       <c r="M28" s="17" t="n"/>
-      <c r="N28" s="19" t="inlineStr">
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O28" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P28" s="17" t="n"/>
+      <c r="P28" s="18" t="n"/>
       <c r="Q28" s="17" t="n"/>
       <c r="R28" s="17" t="n"/>
       <c r="S28" s="17" t="n"/>
@@ -3631,24 +3832,24 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Brands + Categories Module UI</t>
+          <t>Deployment Guide + Work Report + Gantt Update</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Dev 2</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
-        <v>46090</v>
+        <v>46097</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>46096</v>
+        <v>46103</v>
       </c>
       <c r="F29" s="15" t="n">
         <v>1</v>
@@ -3660,13 +3861,13 @@
       <c r="K29" s="17" t="n"/>
       <c r="L29" s="17" t="n"/>
       <c r="M29" s="17" t="n"/>
-      <c r="N29" s="19" t="inlineStr">
+      <c r="N29" s="17" t="n"/>
+      <c r="O29" s="16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O29" s="18" t="n"/>
-      <c r="P29" s="17" t="n"/>
+      <c r="P29" s="18" t="n"/>
       <c r="Q29" s="17" t="n"/>
       <c r="R29" s="17" t="n"/>
       <c r="S29" s="17" t="n"/>
@@ -3674,54 +3875,36 @@
       <c r="U29" s="17" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Vendors Module UI</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Dev 5</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>46090</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-      <c r="K30" s="17" t="n"/>
-      <c r="L30" s="17" t="n"/>
-      <c r="M30" s="17" t="n"/>
-      <c r="N30" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O30" s="18" t="n"/>
-      <c r="P30" s="17" t="n"/>
-      <c r="Q30" s="17" t="n"/>
-      <c r="R30" s="17" t="n"/>
-      <c r="S30" s="17" t="n"/>
-      <c r="T30" s="17" t="n"/>
-      <c r="U30" s="17" t="n"/>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>PHASE 2: CORE MODULES (Mar 24 - Apr 6) — Frontend DONE, Backend in progress</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
+      <c r="L30" s="5" t="n"/>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
+      <c r="O30" s="5" t="n"/>
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="5" t="n"/>
+      <c r="S30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
+      <c r="U30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Zones Module UI</t>
+          <t>Products Module UI (list + forms + 4 tabs)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -3731,17 +3914,17 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Dev 5</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D31" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>46096</v>
+        <v>46103</v>
       </c>
       <c r="F31" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G31" s="17" t="n"/>
       <c r="H31" s="17" t="n"/>
@@ -3755,8 +3938,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O31" s="18" t="n"/>
-      <c r="P31" s="17" t="n"/>
+      <c r="O31" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P31" s="18" t="n"/>
       <c r="Q31" s="17" t="n"/>
       <c r="R31" s="17" t="n"/>
       <c r="S31" s="17" t="n"/>
@@ -3766,7 +3953,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Dealers Module UI</t>
+          <t>Brands + Categories Module UI</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -3776,17 +3963,17 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Dev 6</t>
+          <t>Dev 2</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>46103</v>
+        <v>46096</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" s="17" t="n"/>
       <c r="H32" s="17" t="n"/>
@@ -3800,12 +3987,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O32" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P32" s="17" t="n"/>
+      <c r="O32" s="17" t="n"/>
+      <c r="P32" s="18" t="n"/>
       <c r="Q32" s="17" t="n"/>
       <c r="R32" s="17" t="n"/>
       <c r="S32" s="17" t="n"/>
@@ -3815,7 +3998,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Buyers Module UI</t>
+          <t>Vendors Module UI</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -3825,17 +4008,17 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Dev 2</t>
+          <t>Dev 5</t>
         </is>
       </c>
       <c r="D33" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E33" s="14" t="n">
-        <v>46103</v>
+        <v>46096</v>
       </c>
       <c r="F33" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="17" t="n"/>
       <c r="H33" s="17" t="n"/>
@@ -3849,12 +4032,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O33" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P33" s="17" t="n"/>
+      <c r="O33" s="17" t="n"/>
+      <c r="P33" s="18" t="n"/>
       <c r="Q33" s="17" t="n"/>
       <c r="R33" s="17" t="n"/>
       <c r="S33" s="17" t="n"/>
@@ -3864,7 +4043,7 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Orders Module UI (admin)</t>
+          <t>Zones Module UI</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -3874,17 +4053,17 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Dev 1, Dev 2</t>
+          <t>Dev 5</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
         <v>46090</v>
       </c>
       <c r="E34" s="14" t="n">
-        <v>46103</v>
+        <v>46096</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" s="17" t="n"/>
       <c r="H34" s="17" t="n"/>
@@ -3898,12 +4077,8 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O34" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P34" s="17" t="n"/>
+      <c r="O34" s="17" t="n"/>
+      <c r="P34" s="18" t="n"/>
       <c r="Q34" s="17" t="n"/>
       <c r="R34" s="17" t="n"/>
       <c r="S34" s="17" t="n"/>
@@ -3913,7 +4088,7 @@
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Admin Dashboard (stats + recent orders)</t>
+          <t>Dealers Module UI</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -3923,7 +4098,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 6</t>
         </is>
       </c>
       <c r="D35" s="14" t="n">
@@ -3952,7 +4127,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P35" s="17" t="n"/>
+      <c r="P35" s="18" t="n"/>
       <c r="Q35" s="17" t="n"/>
       <c r="R35" s="17" t="n"/>
       <c r="S35" s="17" t="n"/>
@@ -3962,7 +4137,7 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Coupons Module (both frontends)</t>
+          <t>Buyers Module UI</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -3972,14 +4147,14 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Dev 1</t>
+          <t>Dev 2</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
-        <v>46097</v>
+        <v>46090</v>
       </c>
       <c r="E36" s="14" t="n">
-        <v>46110</v>
+        <v>46103</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>2</v>
@@ -3991,17 +4166,17 @@
       <c r="K36" s="17" t="n"/>
       <c r="L36" s="17" t="n"/>
       <c r="M36" s="17" t="n"/>
-      <c r="N36" s="17" t="n"/>
+      <c r="N36" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="O36" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P36" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="P36" s="18" t="n"/>
       <c r="Q36" s="17" t="n"/>
       <c r="R36" s="17" t="n"/>
       <c r="S36" s="17" t="n"/>
@@ -4011,7 +4186,7 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Admin Users Module (both frontends)</t>
+          <t>Orders Module UI (admin)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -4021,14 +4196,14 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Dev 1</t>
+          <t>Dev 1, Dev 2</t>
         </is>
       </c>
       <c r="D37" s="14" t="n">
-        <v>46097</v>
+        <v>46090</v>
       </c>
       <c r="E37" s="14" t="n">
-        <v>46110</v>
+        <v>46103</v>
       </c>
       <c r="F37" s="15" t="n">
         <v>2</v>
@@ -4040,17 +4215,17 @@
       <c r="K37" s="17" t="n"/>
       <c r="L37" s="17" t="n"/>
       <c r="M37" s="17" t="n"/>
-      <c r="N37" s="17" t="n"/>
+      <c r="N37" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="O37" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P37" s="19" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="P37" s="18" t="n"/>
       <c r="Q37" s="17" t="n"/>
       <c r="R37" s="17" t="n"/>
       <c r="S37" s="17" t="n"/>
@@ -4060,7 +4235,7 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Products File Upload UI (Tech Data Sheet)</t>
+          <t>Admin Dashboard (stats + recent orders)</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -4070,17 +4245,17 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Dev 1</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D38" s="14" t="n">
-        <v>46097</v>
+        <v>46090</v>
       </c>
       <c r="E38" s="14" t="n">
         <v>46103</v>
       </c>
       <c r="F38" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G38" s="17" t="n"/>
       <c r="H38" s="17" t="n"/>
@@ -4089,13 +4264,17 @@
       <c r="K38" s="17" t="n"/>
       <c r="L38" s="17" t="n"/>
       <c r="M38" s="17" t="n"/>
-      <c r="N38" s="17" t="n"/>
+      <c r="N38" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="O38" s="19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P38" s="17" t="n"/>
+      <c r="P38" s="18" t="n"/>
       <c r="Q38" s="17" t="n"/>
       <c r="R38" s="17" t="n"/>
       <c r="S38" s="17" t="n"/>
@@ -4103,29 +4282,29 @@
       <c r="U38" s="17" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Pricing Tiers / Discount Backend</t>
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Coupons Module (both frontends)</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Dev 4</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D39" s="14" t="n">
-        <v>46104</v>
+        <v>46097</v>
       </c>
       <c r="E39" s="14" t="n">
         <v>46110</v>
       </c>
       <c r="F39" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="17" t="n"/>
       <c r="H39" s="17" t="n"/>
@@ -4135,8 +4314,16 @@
       <c r="L39" s="17" t="n"/>
       <c r="M39" s="17" t="n"/>
       <c r="N39" s="17" t="n"/>
-      <c r="O39" s="18" t="n"/>
-      <c r="P39" s="20" t="n"/>
+      <c r="O39" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P39" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q39" s="17" t="n"/>
       <c r="R39" s="17" t="n"/>
       <c r="S39" s="17" t="n"/>
@@ -4144,26 +4331,26 @@
       <c r="U39" s="17" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Payment Integration Backend (Razorpay)</t>
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Admin Users Module (both frontends)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Dev 7</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D40" s="14" t="n">
-        <v>46104</v>
+        <v>46097</v>
       </c>
       <c r="E40" s="14" t="n">
-        <v>46117</v>
+        <v>46110</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>2</v>
@@ -4176,35 +4363,43 @@
       <c r="L40" s="17" t="n"/>
       <c r="M40" s="17" t="n"/>
       <c r="N40" s="17" t="n"/>
-      <c r="O40" s="18" t="n"/>
-      <c r="P40" s="20" t="n"/>
-      <c r="Q40" s="20" t="n"/>
+      <c r="O40" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P40" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q40" s="17" t="n"/>
       <c r="R40" s="17" t="n"/>
       <c r="S40" s="17" t="n"/>
       <c r="T40" s="17" t="n"/>
       <c r="U40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Invoice Generation Backend (PDF)</t>
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Products File Upload UI (Tech Data Sheet)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 1</t>
         </is>
       </c>
       <c r="D41" s="14" t="n">
-        <v>46111</v>
+        <v>46097</v>
       </c>
       <c r="E41" s="14" t="n">
-        <v>46117</v>
+        <v>46103</v>
       </c>
       <c r="F41" s="15" t="n">
         <v>1</v>
@@ -4217,65 +4412,83 @@
       <c r="L41" s="17" t="n"/>
       <c r="M41" s="17" t="n"/>
       <c r="N41" s="17" t="n"/>
-      <c r="O41" s="18" t="n"/>
-      <c r="P41" s="17" t="n"/>
-      <c r="Q41" s="20" t="n"/>
+      <c r="O41" s="19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P41" s="18" t="n"/>
+      <c r="Q41" s="17" t="n"/>
       <c r="R41" s="17" t="n"/>
       <c r="S41" s="17" t="n"/>
       <c r="T41" s="17" t="n"/>
       <c r="U41" s="17" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 3: BUSINESS LOGIC &amp; DASHBOARD (Apr 7 - Apr 20)</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
-      <c r="L42" s="5" t="n"/>
-      <c r="M42" s="5" t="n"/>
-      <c r="N42" s="5" t="n"/>
-      <c r="O42" s="5" t="n"/>
-      <c r="P42" s="5" t="n"/>
-      <c r="Q42" s="5" t="n"/>
-      <c r="R42" s="5" t="n"/>
-      <c r="S42" s="5" t="n"/>
-      <c r="T42" s="5" t="n"/>
-      <c r="U42" s="5" t="n"/>
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Pricing Tiers / Discount Backend</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Dev 4</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="n">
+        <v>46104</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>46110</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="17" t="n"/>
+      <c r="H42" s="17" t="n"/>
+      <c r="I42" s="17" t="n"/>
+      <c r="J42" s="17" t="n"/>
+      <c r="K42" s="17" t="n"/>
+      <c r="L42" s="17" t="n"/>
+      <c r="M42" s="17" t="n"/>
+      <c r="N42" s="17" t="n"/>
+      <c r="O42" s="17" t="n"/>
+      <c r="P42" s="20" t="n"/>
+      <c r="Q42" s="17" t="n"/>
+      <c r="R42" s="17" t="n"/>
+      <c r="S42" s="17" t="n"/>
+      <c r="T42" s="17" t="n"/>
+      <c r="U42" s="17" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Inventory Module UI (stock levels, alerts)</t>
+          <t>Payment Integration Backend (Razorpay)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Dev 5</t>
+          <t>Dev 7</t>
         </is>
       </c>
       <c r="D43" s="14" t="n">
-        <v>46118</v>
+        <v>46104</v>
       </c>
       <c r="E43" s="14" t="n">
-        <v>46124</v>
+        <v>46117</v>
       </c>
       <c r="F43" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G43" s="17" t="n"/>
       <c r="H43" s="17" t="n"/>
@@ -4285,10 +4498,10 @@
       <c r="L43" s="17" t="n"/>
       <c r="M43" s="17" t="n"/>
       <c r="N43" s="17" t="n"/>
-      <c r="O43" s="18" t="n"/>
-      <c r="P43" s="17" t="n"/>
-      <c r="Q43" s="17" t="n"/>
-      <c r="R43" s="21" t="n"/>
+      <c r="O43" s="17" t="n"/>
+      <c r="P43" s="20" t="n"/>
+      <c r="Q43" s="20" t="n"/>
+      <c r="R43" s="17" t="n"/>
       <c r="S43" s="17" t="n"/>
       <c r="T43" s="17" t="n"/>
       <c r="U43" s="17" t="n"/>
@@ -4296,24 +4509,24 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Payment Module UI (Razorpay frontend)</t>
+          <t>Invoice Generation Backend (PDF)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Dev 6</t>
+          <t>Dev 3</t>
         </is>
       </c>
       <c r="D44" s="14" t="n">
-        <v>46118</v>
+        <v>46111</v>
       </c>
       <c r="E44" s="14" t="n">
-        <v>46124</v>
+        <v>46117</v>
       </c>
       <c r="F44" s="15" t="n">
         <v>1</v>
@@ -4326,59 +4539,45 @@
       <c r="L44" s="17" t="n"/>
       <c r="M44" s="17" t="n"/>
       <c r="N44" s="17" t="n"/>
-      <c r="O44" s="18" t="n"/>
-      <c r="P44" s="17" t="n"/>
-      <c r="Q44" s="17" t="n"/>
-      <c r="R44" s="21" t="n"/>
+      <c r="O44" s="17" t="n"/>
+      <c r="P44" s="18" t="n"/>
+      <c r="Q44" s="20" t="n"/>
+      <c r="R44" s="17" t="n"/>
       <c r="S44" s="17" t="n"/>
       <c r="T44" s="17" t="n"/>
       <c r="U44" s="17" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>Invoice Module UI (view/download PDF)</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>Dev 6</t>
-        </is>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>46125</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>46131</v>
-      </c>
-      <c r="F45" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="17" t="n"/>
-      <c r="H45" s="17" t="n"/>
-      <c r="I45" s="17" t="n"/>
-      <c r="J45" s="17" t="n"/>
-      <c r="K45" s="17" t="n"/>
-      <c r="L45" s="17" t="n"/>
-      <c r="M45" s="17" t="n"/>
-      <c r="N45" s="17" t="n"/>
-      <c r="O45" s="18" t="n"/>
-      <c r="P45" s="17" t="n"/>
-      <c r="Q45" s="17" t="n"/>
-      <c r="R45" s="17" t="n"/>
-      <c r="S45" s="21" t="n"/>
-      <c r="T45" s="17" t="n"/>
-      <c r="U45" s="17" t="n"/>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PHASE 3: BUSINESS LOGIC &amp; DASHBOARD (Apr 7 - Apr 20)</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="5" t="n"/>
+      <c r="K45" s="5" t="n"/>
+      <c r="L45" s="5" t="n"/>
+      <c r="M45" s="5" t="n"/>
+      <c r="N45" s="5" t="n"/>
+      <c r="O45" s="5" t="n"/>
+      <c r="P45" s="5" t="n"/>
+      <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
+      <c r="S45" s="5" t="n"/>
+      <c r="T45" s="5" t="n"/>
+      <c r="U45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Admin Dashboard Charts (recharts/chart.js)</t>
+          <t>Inventory Module UI (stock levels, alerts)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -4388,17 +4587,17 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 5</t>
         </is>
       </c>
       <c r="D46" s="14" t="n">
         <v>46118</v>
       </c>
       <c r="E46" s="14" t="n">
-        <v>46131</v>
+        <v>46124</v>
       </c>
       <c r="F46" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" s="17" t="n"/>
       <c r="H46" s="17" t="n"/>
@@ -4408,28 +4607,28 @@
       <c r="L46" s="17" t="n"/>
       <c r="M46" s="17" t="n"/>
       <c r="N46" s="17" t="n"/>
-      <c r="O46" s="18" t="n"/>
-      <c r="P46" s="17" t="n"/>
+      <c r="O46" s="17" t="n"/>
+      <c r="P46" s="18" t="n"/>
       <c r="Q46" s="17" t="n"/>
       <c r="R46" s="21" t="n"/>
-      <c r="S46" s="21" t="n"/>
+      <c r="S46" s="17" t="n"/>
       <c r="T46" s="17" t="n"/>
       <c r="U46" s="17" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Reporting APIs (sales, top products, analytics)</t>
+          <t>Payment Module UI (Razorpay frontend)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Dev 3</t>
+          <t>Dev 6</t>
         </is>
       </c>
       <c r="D47" s="14" t="n">
@@ -4449,8 +4648,8 @@
       <c r="L47" s="17" t="n"/>
       <c r="M47" s="17" t="n"/>
       <c r="N47" s="17" t="n"/>
-      <c r="O47" s="18" t="n"/>
-      <c r="P47" s="17" t="n"/>
+      <c r="O47" s="17" t="n"/>
+      <c r="P47" s="18" t="n"/>
       <c r="Q47" s="17" t="n"/>
       <c r="R47" s="21" t="n"/>
       <c r="S47" s="17" t="n"/>
@@ -4460,27 +4659,27 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Delivery Tracking Backend + UI</t>
+          <t>Invoice Module UI (view/download PDF)</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Dev 7</t>
+          <t>Dev 6</t>
         </is>
       </c>
       <c r="D48" s="14" t="n">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="E48" s="14" t="n">
         <v>46131</v>
       </c>
       <c r="F48" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" s="17" t="n"/>
       <c r="H48" s="17" t="n"/>
@@ -4490,10 +4689,10 @@
       <c r="L48" s="17" t="n"/>
       <c r="M48" s="17" t="n"/>
       <c r="N48" s="17" t="n"/>
-      <c r="O48" s="18" t="n"/>
-      <c r="P48" s="17" t="n"/>
+      <c r="O48" s="17" t="n"/>
+      <c r="P48" s="18" t="n"/>
       <c r="Q48" s="17" t="n"/>
-      <c r="R48" s="21" t="n"/>
+      <c r="R48" s="17" t="n"/>
       <c r="S48" s="21" t="n"/>
       <c r="T48" s="17" t="n"/>
       <c r="U48" s="17" t="n"/>
@@ -4501,27 +4700,27 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Notifications Backend (Email/SMS)</t>
+          <t>Admin Dashboard Charts (recharts/chart.js)</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Dev 4</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D49" s="14" t="n">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="E49" s="14" t="n">
         <v>46131</v>
       </c>
       <c r="F49" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G49" s="17" t="n"/>
       <c r="H49" s="17" t="n"/>
@@ -4531,65 +4730,79 @@
       <c r="L49" s="17" t="n"/>
       <c r="M49" s="17" t="n"/>
       <c r="N49" s="17" t="n"/>
-      <c r="O49" s="18" t="n"/>
-      <c r="P49" s="17" t="n"/>
+      <c r="O49" s="17" t="n"/>
+      <c r="P49" s="18" t="n"/>
       <c r="Q49" s="17" t="n"/>
-      <c r="R49" s="17" t="n"/>
+      <c r="R49" s="21" t="n"/>
       <c r="S49" s="21" t="n"/>
       <c r="T49" s="17" t="n"/>
       <c r="U49" s="17" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 4: POLISH &amp; LAUNCH (Apr 21 - Apr 30) 🚀 DEADLINE</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
-      <c r="L50" s="5" t="n"/>
-      <c r="M50" s="5" t="n"/>
-      <c r="N50" s="5" t="n"/>
-      <c r="O50" s="5" t="n"/>
-      <c r="P50" s="5" t="n"/>
-      <c r="Q50" s="5" t="n"/>
-      <c r="R50" s="5" t="n"/>
-      <c r="S50" s="5" t="n"/>
-      <c r="T50" s="5" t="n"/>
-      <c r="U50" s="5" t="n"/>
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Reporting APIs (sales, top products, analytics)</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Dev 3</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>46118</v>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>46124</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="17" t="n"/>
+      <c r="H50" s="17" t="n"/>
+      <c r="I50" s="17" t="n"/>
+      <c r="J50" s="17" t="n"/>
+      <c r="K50" s="17" t="n"/>
+      <c r="L50" s="17" t="n"/>
+      <c r="M50" s="17" t="n"/>
+      <c r="N50" s="17" t="n"/>
+      <c r="O50" s="17" t="n"/>
+      <c r="P50" s="18" t="n"/>
+      <c r="Q50" s="17" t="n"/>
+      <c r="R50" s="21" t="n"/>
+      <c r="S50" s="17" t="n"/>
+      <c r="T50" s="17" t="n"/>
+      <c r="U50" s="17" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
+          <t>Delivery Tracking Backend + UI</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Dev 1, Dev 6</t>
+          <t>Dev 7</t>
         </is>
       </c>
       <c r="D51" s="14" t="n">
-        <v>46132</v>
+        <v>46118</v>
       </c>
       <c r="E51" s="14" t="n">
-        <v>46138</v>
+        <v>46131</v>
       </c>
       <c r="F51" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="17" t="n"/>
       <c r="H51" s="17" t="n"/>
@@ -4599,35 +4812,35 @@
       <c r="L51" s="17" t="n"/>
       <c r="M51" s="17" t="n"/>
       <c r="N51" s="17" t="n"/>
-      <c r="O51" s="18" t="n"/>
-      <c r="P51" s="17" t="n"/>
+      <c r="O51" s="17" t="n"/>
+      <c r="P51" s="18" t="n"/>
       <c r="Q51" s="17" t="n"/>
-      <c r="R51" s="17" t="n"/>
-      <c r="S51" s="17" t="n"/>
-      <c r="T51" s="22" t="n"/>
+      <c r="R51" s="21" t="n"/>
+      <c r="S51" s="21" t="n"/>
+      <c r="T51" s="17" t="n"/>
       <c r="U51" s="17" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>Reporting Dashboard Charts (frontend)</t>
+          <t>Notifications Backend (Email/SMS)</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Dev 2, Dev 5</t>
+          <t>Dev 4</t>
         </is>
       </c>
       <c r="D52" s="14" t="n">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="E52" s="14" t="n">
-        <v>46138</v>
+        <v>46131</v>
       </c>
       <c r="F52" s="15" t="n">
         <v>1</v>
@@ -4640,69 +4853,55 @@
       <c r="L52" s="17" t="n"/>
       <c r="M52" s="17" t="n"/>
       <c r="N52" s="17" t="n"/>
-      <c r="O52" s="18" t="n"/>
-      <c r="P52" s="17" t="n"/>
+      <c r="O52" s="17" t="n"/>
+      <c r="P52" s="18" t="n"/>
       <c r="Q52" s="17" t="n"/>
       <c r="R52" s="17" t="n"/>
-      <c r="S52" s="17" t="n"/>
-      <c r="T52" s="22" t="n"/>
+      <c r="S52" s="21" t="n"/>
+      <c r="T52" s="17" t="n"/>
       <c r="U52" s="17" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>Responsive Design + Mobile Polish</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>Dev 3</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="n">
-        <v>46132</v>
-      </c>
-      <c r="E53" s="14" t="n">
-        <v>46138</v>
-      </c>
-      <c r="F53" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="17" t="n"/>
-      <c r="H53" s="17" t="n"/>
-      <c r="I53" s="17" t="n"/>
-      <c r="J53" s="17" t="n"/>
-      <c r="K53" s="17" t="n"/>
-      <c r="L53" s="17" t="n"/>
-      <c r="M53" s="17" t="n"/>
-      <c r="N53" s="17" t="n"/>
-      <c r="O53" s="18" t="n"/>
-      <c r="P53" s="17" t="n"/>
-      <c r="Q53" s="17" t="n"/>
-      <c r="R53" s="17" t="n"/>
-      <c r="S53" s="17" t="n"/>
-      <c r="T53" s="22" t="n"/>
-      <c r="U53" s="17" t="n"/>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>PHASE 4: POLISH &amp; LAUNCH (Apr 21 - Apr 30) 🚀 DEADLINE</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="5" t="n"/>
+      <c r="I53" s="5" t="n"/>
+      <c r="J53" s="5" t="n"/>
+      <c r="K53" s="5" t="n"/>
+      <c r="L53" s="5" t="n"/>
+      <c r="M53" s="5" t="n"/>
+      <c r="N53" s="5" t="n"/>
+      <c r="O53" s="5" t="n"/>
+      <c r="P53" s="5" t="n"/>
+      <c r="Q53" s="5" t="n"/>
+      <c r="R53" s="5" t="n"/>
+      <c r="S53" s="5" t="n"/>
+      <c r="T53" s="5" t="n"/>
+      <c r="U53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>Integration Testing (API + UI)</t>
+          <t>Role-based Dashboards (dealer, buyer, vendor)</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>All Devs</t>
+          <t>Dev 1, Dev 6</t>
         </is>
       </c>
       <c r="D54" s="14" t="n">
@@ -4722,8 +4921,8 @@
       <c r="L54" s="17" t="n"/>
       <c r="M54" s="17" t="n"/>
       <c r="N54" s="17" t="n"/>
-      <c r="O54" s="18" t="n"/>
-      <c r="P54" s="17" t="n"/>
+      <c r="O54" s="17" t="n"/>
+      <c r="P54" s="18" t="n"/>
       <c r="Q54" s="17" t="n"/>
       <c r="R54" s="17" t="n"/>
       <c r="S54" s="17" t="n"/>
@@ -4733,24 +4932,24 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Bug Fixes &amp; Performance Optimization</t>
+          <t>Reporting Dashboard Charts (frontend)</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>All Devs</t>
+          <t>Dev 2, Dev 5</t>
         </is>
       </c>
       <c r="D55" s="14" t="n">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="E55" s="14" t="n">
-        <v>46145</v>
+        <v>46138</v>
       </c>
       <c r="F55" s="15" t="n">
         <v>1</v>
@@ -4763,35 +4962,35 @@
       <c r="L55" s="17" t="n"/>
       <c r="M55" s="17" t="n"/>
       <c r="N55" s="17" t="n"/>
-      <c r="O55" s="18" t="n"/>
-      <c r="P55" s="17" t="n"/>
+      <c r="O55" s="17" t="n"/>
+      <c r="P55" s="18" t="n"/>
       <c r="Q55" s="17" t="n"/>
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="17" t="n"/>
-      <c r="T55" s="17" t="n"/>
-      <c r="U55" s="22" t="n"/>
+      <c r="T55" s="22" t="n"/>
+      <c r="U55" s="17" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>UAT + Production Deployment</t>
+          <t>Responsive Design + Mobile Polish</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>All Devs</t>
+          <t>Dev 3</t>
         </is>
       </c>
       <c r="D56" s="14" t="n">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="E56" s="14" t="n">
-        <v>46145</v>
+        <v>46138</v>
       </c>
       <c r="F56" s="15" t="n">
         <v>1</v>
@@ -4804,116 +5003,239 @@
       <c r="L56" s="17" t="n"/>
       <c r="M56" s="17" t="n"/>
       <c r="N56" s="17" t="n"/>
-      <c r="O56" s="18" t="n"/>
-      <c r="P56" s="17" t="n"/>
+      <c r="O56" s="17" t="n"/>
+      <c r="P56" s="18" t="n"/>
       <c r="Q56" s="17" t="n"/>
       <c r="R56" s="17" t="n"/>
       <c r="S56" s="17" t="n"/>
-      <c r="T56" s="17" t="n"/>
-      <c r="U56" s="22" t="n"/>
+      <c r="T56" s="22" t="n"/>
+      <c r="U56" s="17" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="23" t="inlineStr">
-        <is>
-          <t>▲ TODAY (Mar 21, 2026) — 5.7 weeks to deadline</t>
-        </is>
-      </c>
-      <c r="B57" s="24" t="n"/>
-      <c r="C57" s="24" t="n"/>
-      <c r="D57" s="24" t="n"/>
-      <c r="E57" s="24" t="n"/>
-      <c r="F57" s="24" t="n"/>
-      <c r="G57" s="24" t="n"/>
-      <c r="H57" s="24" t="n"/>
-      <c r="I57" s="24" t="n"/>
-      <c r="J57" s="24" t="n"/>
-      <c r="K57" s="24" t="n"/>
-      <c r="L57" s="24" t="n"/>
-      <c r="M57" s="24" t="n"/>
-      <c r="N57" s="24" t="n"/>
-      <c r="O57" s="25" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Integration Testing (API + UI)</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Full Stack</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>All Devs</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="n">
+        <v>46132</v>
+      </c>
+      <c r="E57" s="14" t="n">
+        <v>46138</v>
+      </c>
+      <c r="F57" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="17" t="n"/>
+      <c r="J57" s="17" t="n"/>
+      <c r="K57" s="17" t="n"/>
+      <c r="L57" s="17" t="n"/>
+      <c r="M57" s="17" t="n"/>
+      <c r="N57" s="17" t="n"/>
+      <c r="O57" s="17" t="n"/>
+      <c r="P57" s="18" t="n"/>
+      <c r="Q57" s="17" t="n"/>
+      <c r="R57" s="17" t="n"/>
+      <c r="S57" s="17" t="n"/>
+      <c r="T57" s="22" t="n"/>
+      <c r="U57" s="17" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Bug Fixes &amp; Performance Optimization</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Full Stack</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>All Devs</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E58" s="14" t="n">
+        <v>46145</v>
+      </c>
+      <c r="F58" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="17" t="n"/>
+      <c r="H58" s="17" t="n"/>
+      <c r="I58" s="17" t="n"/>
+      <c r="J58" s="17" t="n"/>
+      <c r="K58" s="17" t="n"/>
+      <c r="L58" s="17" t="n"/>
+      <c r="M58" s="17" t="n"/>
+      <c r="N58" s="17" t="n"/>
+      <c r="O58" s="17" t="n"/>
+      <c r="P58" s="18" t="n"/>
+      <c r="Q58" s="17" t="n"/>
+      <c r="R58" s="17" t="n"/>
+      <c r="S58" s="17" t="n"/>
+      <c r="T58" s="17" t="n"/>
+      <c r="U58" s="22" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>UAT + Production Deployment</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Full Stack</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>All Devs</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E59" s="14" t="n">
+        <v>46145</v>
+      </c>
+      <c r="F59" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="17" t="n"/>
+      <c r="H59" s="17" t="n"/>
+      <c r="I59" s="17" t="n"/>
+      <c r="J59" s="17" t="n"/>
+      <c r="K59" s="17" t="n"/>
+      <c r="L59" s="17" t="n"/>
+      <c r="M59" s="17" t="n"/>
+      <c r="N59" s="17" t="n"/>
+      <c r="O59" s="17" t="n"/>
+      <c r="P59" s="18" t="n"/>
+      <c r="Q59" s="17" t="n"/>
+      <c r="R59" s="17" t="n"/>
+      <c r="S59" s="17" t="n"/>
+      <c r="T59" s="17" t="n"/>
+      <c r="U59" s="22" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>▲ TODAY (Mar 23, 2026) — 5.4 weeks to deadline</t>
+        </is>
+      </c>
+      <c r="B60" s="24" t="n"/>
+      <c r="C60" s="24" t="n"/>
+      <c r="D60" s="24" t="n"/>
+      <c r="E60" s="24" t="n"/>
+      <c r="F60" s="24" t="n"/>
+      <c r="G60" s="24" t="n"/>
+      <c r="H60" s="24" t="n"/>
+      <c r="I60" s="24" t="n"/>
+      <c r="J60" s="24" t="n"/>
+      <c r="K60" s="24" t="n"/>
+      <c r="L60" s="24" t="n"/>
+      <c r="M60" s="24" t="n"/>
+      <c r="N60" s="24" t="n"/>
+      <c r="O60" s="24" t="n"/>
+      <c r="P60" s="25" t="inlineStr">
         <is>
           <t>▲ NOW</t>
         </is>
       </c>
-      <c r="P57" s="24" t="n"/>
-      <c r="Q57" s="24" t="n"/>
-      <c r="R57" s="24" t="n"/>
-      <c r="S57" s="24" t="n"/>
-      <c r="T57" s="24" t="n"/>
-      <c r="U57" s="24" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="26" t="inlineStr">
+      <c r="Q60" s="24" t="n"/>
+      <c r="R60" s="24" t="n"/>
+      <c r="S60" s="24" t="n"/>
+      <c r="T60" s="24" t="n"/>
+      <c r="U60" s="24" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="26" t="inlineStr">
         <is>
           <t>LEGEND:</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="27" t="n"/>
-      <c r="B60" s="28" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="27" t="n"/>
+      <c r="B63" s="28" t="inlineStr">
         <is>
           <t>Completed (Jan 22 - Mar 10)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="29" t="n"/>
-      <c r="B61" s="28" t="inlineStr">
-        <is>
-          <t>Phase 1: Foundation (Mar 10-23) — 100% DONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="30" t="n"/>
-      <c r="B62" s="28" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="29" t="n"/>
+      <c r="B64" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1: Foundation (Mar 10-21) — 100% DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="30" t="n"/>
+      <c r="B65" s="28" t="inlineStr">
         <is>
           <t>Phase 2: Core CRUD (Mar 24 - Apr 6) — frontend DONE, backend: Razorpay/Invoice/Pricing pending</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="31" t="n"/>
-      <c r="B63" s="28" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="31" t="n"/>
+      <c r="B66" s="28" t="inlineStr">
         <is>
           <t>Phase 3: Business Logic &amp; Dashboard (Apr 7-20)</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="32" t="n"/>
-      <c r="B64" s="28" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="32" t="n"/>
+      <c r="B67" s="28" t="inlineStr">
         <is>
           <t>Phase 4: Polish &amp; Launch (Apr 21-30)</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="33" t="n"/>
-      <c r="B65" s="28" t="inlineStr">
-        <is>
-          <t>TODAY marker (Mar 21)</t>
+    <row r="68">
+      <c r="A68" s="33" t="n"/>
+      <c r="B68" s="28" t="inlineStr">
+        <is>
+          <t>TODAY marker (Mar 23)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A53:U53"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A50:U50"/>
-    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="A30:U30"/>
+    <mergeCell ref="A60:F60"/>
     <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B67:D67"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:U5"/>
-    <mergeCell ref="A42:U42"/>
+    <mergeCell ref="A45:U45"/>
     <mergeCell ref="B65:D65"/>
     <mergeCell ref="A14:U14"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="A27:U27"/>
+    <mergeCell ref="B68:D68"/>
     <mergeCell ref="B64:D64"/>
-    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4925,7 +5247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4943,7 +5265,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Start: 22 Jan 2026  |  Today: 21 Mar 2026  |  Deadline: 30 Apr 2026</t>
+          <t>Start: 22 Jan 2026  |  Today: 23 Mar 2026  |  Deadline: 30 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -4982,12 +5304,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>21 Mar 2026</t>
+          <t>23 Mar 2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>8 weeks elapsed</t>
+          <t>9 weeks elapsed</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5326,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>5.7 weeks remaining</t>
+          <t>5.4 weeks remaining</t>
         </is>
       </c>
     </row>
@@ -5055,12 +5377,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>21 modules</t>
+          <t>24 modules</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Auth, Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Cart, Wishlist, Coupon, Admin Users, Address, Schema, Seed, Validation, RBAC, Pagination, File Upload, Order State Machine, Inventory</t>
+          <t>Auth, Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Cart, Wishlist, Coupon, Admin Users, Address, Schema, Seed, Validation, RBAC, Pagination, File Upload, Order State Machine, Inventory, Back-order Logic, Auto-entity Creation</t>
         </is>
       </c>
     </row>
@@ -5106,12 +5428,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>54 items</t>
+          <t>57 items</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>All admin CRUD (11 modules incl. Coupons &amp; Admin Users), all storefront pages (11), buyer account (4), foundation (10), UI components (4), file upload UI, nav/footer</t>
+          <t>All admin CRUD (11 modules incl. Coupons &amp; Admin Users), all storefront pages (11), buyer account (4), foundation (10), UI components (4), file upload UI, nav/footer, logo branding, token auto-refresh</t>
         </is>
       </c>
     </row>
@@ -5133,415 +5455,432 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="35" t="inlineStr"/>
-      <c r="B17" s="35" t="inlineStr"/>
-      <c r="C17" s="35" t="inlineStr"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>3 items</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Deployment Guide, Daily Work Report, Gantt Chart — all completed</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="37" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr"/>
+      <c r="B18" s="35" t="inlineStr"/>
+      <c r="C18" s="35" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>Overall Completion</t>
         </is>
       </c>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>~70%</t>
-        </is>
-      </c>
-      <c r="C18" s="38" t="inlineStr">
-        <is>
-          <t>Phase 1 100% done. Phase 2 frontend done. Remaining: 4 backend features + 7 frontend UIs + testing/deployment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="35" t="inlineStr"/>
-      <c r="B19" s="35" t="inlineStr"/>
-      <c r="C19" s="35" t="inlineStr"/>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>~72%</t>
+        </is>
+      </c>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>Phase 1 100% done. Phase 2 frontend done. All bug fixes resolved. Remaining: 4 backend features + 7 frontend UIs + testing/deployment.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="A20" s="35" t="inlineStr"/>
+      <c r="B20" s="35" t="inlineStr"/>
+      <c r="C20" s="35" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>RISK ASSESSMENT</t>
         </is>
       </c>
-      <c r="B20" s="36" t="inlineStr"/>
-      <c r="C20" s="36" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Schedule Risk</t>
-        </is>
-      </c>
-      <c r="B21" s="39" t="inlineStr">
-        <is>
-          <t>LOW-MEDIUM</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Ahead of schedule. Phase 1 fully done. ~30% work in 5.7 weeks. Comfortable pace.</t>
-        </is>
-      </c>
+      <c r="B21" s="36" t="inlineStr"/>
+      <c r="C21" s="36" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Critical Path</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Razorpay + Invoice PDF</t>
+          <t>Schedule Risk</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>LOW-MEDIUM</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Payment backend needed before Payment UI; Invoice backend needed before Invoice UI</t>
+          <t>Ahead of schedule. Phase 1 fully done. ~28% work in 5.4 weeks. Comfortable pace.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Parallel Tracks Needed</t>
+          <t>Critical Path</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Razorpay + Invoice PDF</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Backend (Razorpay, Invoice, Reporting) + Frontend (Inventory UI, Charts) simultaneously</t>
+          <t>Payment backend needed before Payment UI; Invoice backend needed before Invoice UI</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>Parallel Tracks Needed</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Backend (Razorpay, Invoice, Reporting) + Frontend (Inventory UI, Charts) simultaneously</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>Recommended Action</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>START PHASE 2 BACKEND</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Begin Razorpay integration and Invoice PDF generation next week</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="35" t="inlineStr"/>
-      <c r="B25" s="35" t="inlineStr"/>
-      <c r="C25" s="35" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="36" t="inlineStr">
+      <c r="A26" s="35" t="inlineStr"/>
+      <c r="B26" s="35" t="inlineStr"/>
+      <c r="C26" s="35" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
         <is>
           <t>PHASE PLAN (REMAINING)</t>
         </is>
       </c>
-      <c r="B26" s="36" t="inlineStr">
+      <c r="B27" s="36" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="C26" s="36" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>Focus</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>COMPLETED ✅</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>All items done: Pagination, File Upload, Order State Machine, Inventory Decrement</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Phase 2 Remaining</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Mar 24 - Apr 6 (2 wks)</t>
+          <t>COMPLETED ✅</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation</t>
+          <t>All items done: Pagination, File Upload, Order State Machine, Inventory Decrement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Phase 3: Business Logic</t>
+          <t>Phase 2 Remaining</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Apr 7-20 (2 wks)</t>
+          <t>Mar 24 - Apr 6 (2 wks)</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Inventory UI, Payment UI, Invoice UI, Dashboard charts, Reporting APIs, Delivery tracking, Notifications</t>
+          <t>Pricing tiers, Razorpay payment backend, Invoice PDF generation</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t>Phase 3: Business Logic</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Apr 7-20 (2 wks)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Inventory UI, Payment UI, Invoice UI, Dashboard charts, Reporting APIs, Delivery tracking, Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>Phase 4: Polish &amp; Launch</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Apr 21-30 (1.5 wks)</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Role-based dashboards, responsive design, testing, UAT, deployment</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="35" t="inlineStr"/>
-      <c r="B31" s="35" t="inlineStr"/>
-      <c r="C31" s="35" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="36" t="inlineStr">
+      <c r="A32" s="35" t="inlineStr"/>
+      <c r="B32" s="35" t="inlineStr"/>
+      <c r="C32" s="35" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
         <is>
           <t>WHAT WAS DONE AHEAD OF SCHEDULE</t>
         </is>
       </c>
-      <c r="B32" s="36" t="inlineStr"/>
-      <c r="C32" s="36" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>All Admin CRUD UIs (11 modules)</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Phase 2 → Done in Phase 1</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard, Coupons, Admin Users</t>
-        </is>
-      </c>
+      <c r="B33" s="36" t="inlineStr"/>
+      <c r="C33" s="36" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>All Storefront Pages (11 pages)</t>
+          <t>All Admin CRUD UIs (11 modules)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Phase 2-3 → Done in Phase 1</t>
+          <t>Phase 2 → Done in Phase 1</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Home, Products, Detail, Cart, Checkout, Confirmation, Categories, About, Contact + Header/Footer</t>
+          <t>Products, Brands, Categories, Vendors, Zones, Buyers, Dealers, Orders, Dashboard, Coupons, Admin Users</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Buyer Account (4 pages)</t>
+          <t>All Storefront Pages (11 pages)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Phase 3 → Done in Phase 1</t>
+          <t>Phase 2-3 → Done in Phase 1</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>My Account, My Orders, Addresses, Wishlist</t>
+          <t>Home, Products, Detail, Cart, Checkout, Confirmation, Categories, About, Contact + Header/Footer</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Cart + Wishlist + Coupon APIs</t>
+          <t>Buyer Account (4 pages)</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Not in plan → Done</t>
+          <t>Phase 3 → Done in Phase 1</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Server-side cart, wishlist, coupon validation — bonus features</t>
+          <t>My Account, My Orders, Addresses, Wishlist</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Phase 1 Backend (4 items)</t>
+          <t>Cart + Wishlist + Coupon APIs</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Done on time (Mar 17)</t>
+          <t>Not in plan → Done</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Pagination, Multer upload, Order state machine, Inventory decrement</t>
+          <t>Server-side cart, wishlist, coupon validation — bonus features</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t>Phase 1 Backend (4 items)</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Done on time (Mar 17)</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Pagination, Multer upload, Order state machine, Inventory decrement</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>Coupons + Admin Users (legacy admin)</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Done Mar 21</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Full CRUD modules added to both React frontend and legacy admin panel</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="35" t="inlineStr"/>
-      <c r="B39" s="35" t="inlineStr"/>
-      <c r="C39" s="35" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="36" t="inlineStr">
+      <c r="A40" s="35" t="inlineStr"/>
+      <c r="B40" s="35" t="inlineStr"/>
+      <c r="C40" s="35" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="36" t="inlineStr">
         <is>
           <t>TEAM ALLOCATION (suggested for remaining)</t>
         </is>
       </c>
-      <c r="B40" s="36" t="inlineStr"/>
-      <c r="C40" s="36" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Dev 1 (Frontend Lead)</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr"/>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Inventory UI → Role-based Dashboards → Responsive polish</t>
-        </is>
-      </c>
+      <c r="B41" s="36" t="inlineStr"/>
+      <c r="C41" s="36" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Dev 2 (Frontend)</t>
+          <t>Dev 1 (Frontend Lead)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr"/>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Dashboard Charts → Reporting UI → Integration testing</t>
+          <t>Inventory UI → Role-based Dashboards → Responsive polish</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Dev 3 (Backend + Frontend)</t>
+          <t>Dev 2 (Frontend)</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Invoice PDF backend → Reporting APIs → Invoice UI</t>
+          <t>Dashboard Charts → Reporting UI → Integration testing</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Dev 4 (Backend Lead)</t>
+          <t>Dev 3 (Backend + Frontend)</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr"/>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Pricing Tiers → Notifications (Email/SMS)</t>
+          <t>Invoice PDF backend → Reporting APIs → Invoice UI</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Dev 5 (Frontend)</t>
+          <t>Dev 4 (Backend Lead)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr"/>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Dashboard Charts → Responsive design</t>
+          <t>Pricing Tiers → Notifications (Email/SMS)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Dev 6 (Frontend)</t>
+          <t>Dev 5 (Frontend)</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr"/>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Payment UI → Invoice UI → Role-based views</t>
+          <t>Dashboard Charts → Responsive design</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Dev 7 (Backend)</t>
+          <t>Dev 6 (Frontend)</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr"/>
       <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Payment UI → Invoice UI → Role-based views</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Dev 7 (Backend)</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr"/>
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Razorpay integration → Delivery tracking backend + UI</t>
         </is>

</xml_diff>